<commit_message>
Fix unit errors: FX-convert foreign mcap, P/B artifacts, penny momentum
Audit-driven unit/aesthetic fixes:
- FOREIGN MCAP was shown in LOCAL CURRENCY as if USD across every sheet (not
  just Global Picks): Samsung read "$1.87 quadrillion" (₩), FPT.VN's $5B co
  bucketed "large". Now FX-converted to USD at the source in unified_score
  (mcap_m + mcap_bucket both correct everywhere); Samsung -> $1.37T, FPT -> $4.7B
  mid. Removed the now-double-counting FX call in Global Picks.
- P/B ARTIFACTS: tightened the guard 100 -> 30 on both the yfinance and SEC paths
  (TSM "98x" is an ADR currency mismatch; real ~7x). 54 -> 0 bogus P/B.
- PENNY MOMENTUM: build_price_stats now skips sub-$1 stocks whose % moves are
  noise (ARDS $0.003 -> "+1450%"). Biggest-mover is now a real name (MRVL +271%).

validate clean (0 failures); no absurd mcaps in the pick sheets.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzLWQfQoCmwwwE2QTFQZro
</commit_message>
<xml_diff>
--- a/people_monitor.xlsx
+++ b/people_monitor.xlsx
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>40.8</v>
+        <v>40.7</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>1.8</v>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D31" s="11" t="n">
         <v>1.2</v>
@@ -2041,98 +2041,98 @@
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>DFS.L</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>TPG Inc.</t>
+          <t>DFS Furniture plc</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="D36" s="11" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="E36" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>Dominic Picone</t>
+          <t>Tony Buffin</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>NGVT</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Ingevity Corporation</t>
+          <t>TPG Inc.</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="E37" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>Daniel Sansone</t>
+          <t>Dominic Picone</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>REI</t>
+          <t>NGVT</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Ring Energy, Inc.</t>
+          <t>Ingevity Corporation</t>
         </is>
       </c>
       <c r="C38" s="11" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="D38" s="11" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E38" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>David Habachy</t>
+          <t>Daniel Sansone</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
@@ -2142,33 +2142,33 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>WMG</t>
+          <t>REI</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Warner Music Group Corp.</t>
+          <t>Ring Energy, Inc.</t>
         </is>
       </c>
       <c r="C39" s="11" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="E39" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>Len Blavatnik</t>
+          <t>David Habachy</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
@@ -2178,33 +2178,33 @@
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>WMG</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>MP Materials Corp.</t>
+          <t>Warner Music Group Corp.</t>
         </is>
       </c>
       <c r="C40" s="11" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="D40" s="11" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="E40" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>Randall Weisenburger</t>
+          <t>Len Blavatnik</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
@@ -2214,33 +2214,33 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Innoviva, Inc.</t>
+          <t>Harbour Energy plc</t>
         </is>
       </c>
       <c r="C41" s="11" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="E41" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>Mark DiPaolo</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
@@ -2250,33 +2250,33 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>AGEN</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Agenus Inc.</t>
+          <t>MP Materials Corp.</t>
         </is>
       </c>
       <c r="C42" s="11" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="D42" s="11" t="n">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="E42" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>Brian Corvese</t>
+          <t>Randall Weisenburger</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
@@ -2286,33 +2286,33 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>DFS.L</t>
+          <t>INVA</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>DFS Furniture plc</t>
+          <t>Innoviva, Inc.</t>
         </is>
       </c>
       <c r="C43" s="11" t="n">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="E43" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>Tony Buffin</t>
+          <t>Mark DiPaolo</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
@@ -2322,91 +2322,91 @@
       </c>
       <c r="H43" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>PMTR</t>
+          <t>AGEN</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Perimeter Acquisition Corp</t>
+          <t>Agenus Inc.</t>
         </is>
       </c>
       <c r="C44" s="11" t="n">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="D44" s="11" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="E44" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>Jack Selby</t>
+          <t>Brian Corvese</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>ADAG</t>
+          <t>PMTR</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Adagene Inc.</t>
+          <t>Perimeter Acquisition Corp</t>
         </is>
       </c>
       <c r="C45" s="11" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="D45" s="11" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E45" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>Li Li</t>
+          <t>Jack Selby</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>ADAG</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holdi</t>
+          <t>Adagene Inc.</t>
         </is>
       </c>
       <c r="C46" s="11" t="n">
@@ -2420,33 +2420,33 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>Poh Kiong Tan</t>
+          <t>Li Li</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>SKF-B.ST</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>AB SKF (publ)</t>
+          <t>Trident Digital Tech Holdi</t>
         </is>
       </c>
       <c r="C47" s="11" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="D47" s="11" t="n">
         <v>0</v>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Hock Goh</t>
+          <t>Poh Kiong Tan</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
@@ -2466,254 +2466,254 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>SKF-B.ST</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>ConocoPhillips</t>
+          <t>AB SKF (publ)</t>
         </is>
       </c>
       <c r="C48" s="11" t="n">
-        <v>3.8</v>
+        <v>4.9</v>
       </c>
       <c r="D48" s="11" t="n">
-        <v>6.1</v>
+        <v>0</v>
       </c>
       <c r="E48" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>Sharmila Mulligan</t>
+          <t>Hock Goh</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>SSYS</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Stratasys Ltd.</t>
+          <t>ConocoPhillips</t>
         </is>
       </c>
       <c r="C49" s="11" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>0.5</v>
+        <v>6.1</v>
       </c>
       <c r="E49" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>Aris Kekedjian</t>
+          <t>Sharmila Mulligan</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>SSYS</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Sierra Bancorp</t>
+          <t>Stratasys Ltd.</t>
         </is>
       </c>
       <c r="C50" s="11" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="D50" s="11" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="E50" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>Laurence Dutto</t>
+          <t>Aris Kekedjian</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>BSRR</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>TotalEnergies SE</t>
+          <t>Sierra Bancorp</t>
         </is>
       </c>
       <c r="C51" s="11" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="D51" s="11" t="n">
-        <v>3.2</v>
+        <v>0.1</v>
       </c>
       <c r="E51" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>Anelise Lara</t>
+          <t>Laurence Dutto</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Lands' End, Inc.</t>
+          <t>TotalEnergies SE</t>
         </is>
       </c>
       <c r="C52" s="11" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D52" s="11" t="n">
         <v>3.2</v>
-      </c>
-      <c r="D52" s="11" t="n">
-        <v>1.9</v>
       </c>
       <c r="E52" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>Josephine Linden</t>
+          <t>Anelise Lara</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Commercial Metals Company</t>
+          <t>Lands' End, Inc.</t>
         </is>
       </c>
       <c r="C53" s="11" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="D53" s="11" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E53" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>John McPherson</t>
+          <t>Josephine Linden</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>SIMO</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Silicon Motion Technology </t>
+          <t>Semtech Corporation</t>
         </is>
       </c>
       <c r="C54" s="11" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="E54" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>Steve Chen</t>
+          <t>Sylvia Summers</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
@@ -2725,31 +2725,31 @@
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>0086.HK</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Porch Group, Inc.</t>
+          <t>Sun Hung Kai &amp; Co. Limited</t>
         </is>
       </c>
       <c r="C55" s="11" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D55" s="11" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E55" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>Amanda Reierson</t>
+          <t>Jacqueline Leung</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H55" s="10" t="inlineStr">
@@ -2761,26 +2761,26 @@
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Amprius Technologies, Inc.</t>
+          <t>Commercial Metals Company</t>
         </is>
       </c>
       <c r="C56" s="11" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="D56" s="11" t="n">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="E56" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>Donald Dixon</t>
+          <t>John McPherson</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
@@ -2797,31 +2797,31 @@
     <row r="57" ht="14" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>SIMO</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Semtech Corporation</t>
+          <t xml:space="preserve">Silicon Motion Technology </t>
         </is>
       </c>
       <c r="C57" s="11" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>2.2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>Sylvia Summers</t>
+          <t>Steve Chen</t>
         </is>
       </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="H57" s="10" t="inlineStr">
@@ -2833,31 +2833,31 @@
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>HLI</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Houlihan Lokey, Inc.</t>
+          <t>Porch Group, Inc.</t>
         </is>
       </c>
       <c r="C58" s="11" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="D58" s="11" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="E58" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>Tommaso Lillo</t>
+          <t>Amanda Reierson</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
@@ -2869,26 +2869,26 @@
     <row r="59" ht="14" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>AMPX</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy plc</t>
+          <t>Amprius Technologies, Inc.</t>
         </is>
       </c>
       <c r="C59" s="11" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="D59" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E59" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>Donald Dixon</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
@@ -2898,131 +2898,131 @@
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>RLXXF</t>
+          <t>HLI</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>RELX PLC</t>
+          <t>Houlihan Lokey, Inc.</t>
         </is>
       </c>
       <c r="C60" s="11" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="D60" s="11" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="E60" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>Suzanne Wood</t>
+          <t>Tommaso Lillo</t>
         </is>
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>UBSI</t>
+          <t>RLXXF</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>United Bankshares, Inc.</t>
+          <t>RELX PLC</t>
         </is>
       </c>
       <c r="C61" s="11" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="D61" s="11" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="E61" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>J. Mcnamara,Michael Fitzgerald</t>
+          <t>Suzanne Wood</t>
         </is>
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>UBSI</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Danaos Corporation</t>
+          <t>United Bankshares, Inc.</t>
         </is>
       </c>
       <c r="C62" s="11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D62" s="11" t="n">
         <v>1.4</v>
       </c>
-      <c r="D62" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E62" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>Dimitris Vastarouchas</t>
+          <t>J. Mcnamara,Michael Fitzgerald</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>EVR</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Evercore Inc.</t>
+          <t>Danaos Corporation</t>
         </is>
       </c>
       <c r="C63" s="11" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="D63" s="11" t="n">
         <v>1</v>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Knee</t>
+          <t>Dimitris Vastarouchas</t>
         </is>
       </c>
       <c r="G63" s="10" t="inlineStr">
@@ -3042,69 +3042,69 @@
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>EVR</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Telefônica Brasil S.A.</t>
+          <t>Evercore Inc.</t>
         </is>
       </c>
       <c r="C64" s="11" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="D64" s="11" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>Peter Loscher</t>
+          <t>Jonathan Knee</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>VIV</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group Ltd</t>
+          <t>Telefônica Brasil S.A.</t>
         </is>
       </c>
       <c r="C65" s="11" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="D65" s="11" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E65" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>Peter Loscher</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
@@ -3114,33 +3114,33 @@
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>United Microelectronics Co</t>
+          <t>Woodside Energy Group Ltd</t>
         </is>
       </c>
       <c r="C66" s="11" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="D66" s="11" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="E66" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>Jason Wang</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
@@ -3150,33 +3150,33 @@
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Star Bulk Carriers Corp.</t>
+          <t>United Microelectronics Co</t>
         </is>
       </c>
       <c r="C67" s="11" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D67" s="11" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="E67" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>Raffaele Zagari</t>
+          <t>Jason Wang</t>
         </is>
       </c>
       <c r="G67" s="10" t="inlineStr">
@@ -3186,74 +3186,74 @@
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>SASOF</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Sasol Limited</t>
+          <t>Star Bulk Carriers Corp.</t>
         </is>
       </c>
       <c r="C68" s="11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D68" s="11" t="n">
-        <v>0.3</v>
+        <v>1.7</v>
       </c>
       <c r="E68" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>Vuyo Kahla</t>
+          <t>Raffaele Zagari</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>CENX</t>
+          <t>SASOF</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Century Aluminum Company</t>
+          <t>Sasol Limited</t>
         </is>
       </c>
       <c r="C69" s="11" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D69" s="11" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="E69" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>Andrew Michelmore</t>
+          <t>Vuyo Kahla</t>
         </is>
       </c>
       <c r="G69" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="H69" s="10" t="inlineStr">
@@ -3265,26 +3265,26 @@
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>EIPAF</t>
+          <t>CENX</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Eni S.p.A.</t>
+          <t>Century Aluminum Company</t>
         </is>
       </c>
       <c r="C70" s="11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D70" s="11" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="E70" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>Massimo Belcredi</t>
+          <t>Andrew Michelmore</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
@@ -3294,19 +3294,19 @@
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>KEN</t>
+          <t>EIPAF</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Kenon Holdings Ltd.</t>
+          <t>Eni S.p.A.</t>
         </is>
       </c>
       <c r="C71" s="11" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>Aviad Kaufman</t>
+          <t>Massimo Belcredi</t>
         </is>
       </c>
       <c r="G71" s="10" t="inlineStr">
@@ -3330,69 +3330,69 @@
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>WIT</t>
+          <t>KEN</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Wipro Limited</t>
+          <t>Kenon Holdings Ltd.</t>
         </is>
       </c>
       <c r="C72" s="11" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D72" s="11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E72" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>Rishad Premji</t>
+          <t>Aviad Kaufman</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>ADDYY</t>
+          <t>WIT</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>adidas AG</t>
+          <t>Wipro Limited</t>
         </is>
       </c>
       <c r="C73" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="11" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E73" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>Nassef Sawiris</t>
+          <t>Rishad Premji</t>
         </is>
       </c>
       <c r="G73" s="10" t="inlineStr">
@@ -3402,19 +3402,19 @@
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>UPMMY</t>
+          <t>ADDYY</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>UPM-Kymmene Oyj</t>
+          <t>adidas AG</t>
         </is>
       </c>
       <c r="C74" s="11" t="n">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Henrik Ehrnrooth</t>
+          <t>Nassef Sawiris</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
@@ -3438,19 +3438,19 @@
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>0001.HK</t>
+          <t>UPMMY</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>CK Hutchison Holdings Limi</t>
+          <t>UPM-Kymmene Oyj</t>
         </is>
       </c>
       <c r="C75" s="11" t="n">
@@ -3464,29 +3464,29 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>Kwai Wong</t>
+          <t>Henrik Ehrnrooth</t>
         </is>
       </c>
       <c r="G75" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>0086.HK</t>
+          <t>0001.HK</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Sun Hung Kai &amp; Co. Limited</t>
+          <t>CK Hutchison Holdings Limi</t>
         </is>
       </c>
       <c r="C76" s="11" t="n">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>Jacqueline Leung</t>
+          <t>Kwai Wong</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="H76" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
         </is>
       </c>
       <c r="C82" s="11" t="n">
-        <v>-2.7</v>
+        <v>-2.6</v>
       </c>
       <c r="D82" s="11" t="n">
         <v>5.2</v>
@@ -5980,7 +5980,7 @@
         </is>
       </c>
       <c r="F5" s="11" t="n">
-        <v>40.8</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
@@ -7420,7 +7420,7 @@
         </is>
       </c>
       <c r="F53" s="11" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
@@ -7480,7 +7480,7 @@
         </is>
       </c>
       <c r="F55" s="11" t="n">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
@@ -7636,72 +7636,72 @@
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Dominic Picone</t>
+          <t>Tony Buffin</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>DFS Furniture</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>PE/Buyout</t>
+          <t>Public Company</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>DFS.L</t>
         </is>
       </c>
       <c r="F61" s="11" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Allan D. Schoening</t>
+          <t>Dominic Picone</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Civeo</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Public Company</t>
+          <t>PE/Buyout</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>CVEO</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="F62" s="11" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Daniel Sansone</t>
+          <t>Allan D. Schoening</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Ingevity</t>
+          <t>Civeo</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -7716,22 +7716,22 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>NGVT</t>
+          <t>CVEO</t>
         </is>
       </c>
       <c r="F63" s="11" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>David Habachy</t>
+          <t>Daniel Sansone</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Ring Energy</t>
+          <t>Ingevity</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -7746,22 +7746,22 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>REI</t>
+          <t>NGVT</t>
         </is>
       </c>
       <c r="F64" s="11" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Pam Kaufman</t>
+          <t>David Habachy</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Paramount Skydance</t>
+          <t>Ring Energy</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -7776,22 +7776,22 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>PSKY</t>
+          <t>REI</t>
         </is>
       </c>
       <c r="F65" s="11" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Len Blavatnik</t>
+          <t>Pam Kaufman</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Warner Music Group</t>
+          <t>Paramount Skydance</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>WMG</t>
+          <t>PSKY</t>
         </is>
       </c>
       <c r="F66" s="11" t="n">
@@ -7816,12 +7816,12 @@
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Randall Weisenburger</t>
+          <t>Len Blavatnik</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>MP Materials</t>
+          <t>Warner Music Group</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -7836,22 +7836,22 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>WMG</t>
         </is>
       </c>
       <c r="F67" s="11" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>Mark DiPaolo</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Innoviva</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -7866,22 +7866,22 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F68" s="11" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Randle Reece</t>
+          <t>Alexander Krane</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>AMN Healthcare Services</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -7896,22 +7896,22 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>AMN</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F69" s="11" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>Tim Cahill</t>
+          <t>Andrea Pinarel</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Lockheed Martin</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -7926,22 +7926,22 @@
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F70" s="11" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>Robert Colligan</t>
+          <t>David Kennedy</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Dynex Capital</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -7951,27 +7951,27 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F71" s="11" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>Brian Corvese</t>
+          <t>Feyyaz Etiz</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Agenus</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -7986,22 +7986,22 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>AGEN</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F72" s="11" t="n">
-        <v>6.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>David Moradi</t>
+          <t>Gustavo Baquero</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>AudioEye</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -8016,22 +8016,22 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F73" s="11" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>Tiago Miranda</t>
+          <t>Linda Cook</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Atlas Lithium</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -8046,22 +8046,22 @@
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>ATLX</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F74" s="11" t="n">
-        <v>6.1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>Charles Leykum</t>
+          <t>Michael Tuffin</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Talon Capital (SPAC</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -8076,22 +8076,22 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>TLNC</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F75" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Tony Buffin</t>
+          <t>Nathan Mauzy</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>DFS Furniture</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -8106,22 +8106,22 @@
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>DFS.L</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F76" s="11" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>Paul Allen</t>
+          <t>Randall Weisenburger</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Airship AI Holdings</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -8136,22 +8136,22 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="F77" s="11" t="n">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>David Allen</t>
+          <t>Mark DiPaolo</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>Innoviva</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -8166,22 +8166,22 @@
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>INVA</t>
         </is>
       </c>
       <c r="F78" s="11" t="n">
-        <v>5.5</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>Laura Duda</t>
+          <t>Randle Reece</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>The Goodyear Tire &amp; Rubber</t>
+          <t>AMN Healthcare Services</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -8196,22 +8196,22 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>AMN</t>
         </is>
       </c>
       <c r="F79" s="11" t="n">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>Oscar Iglesias</t>
+          <t>Tim Cahill</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Codere Online Luxembourg</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -8226,22 +8226,22 @@
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>CDROW</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="F80" s="11" t="n">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Martin Bork</t>
+          <t>Robert Colligan</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Navigator Holdings</t>
+          <t>Dynex Capital</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -8251,27 +8251,27 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>NVGS</t>
+          <t>DX</t>
         </is>
       </c>
       <c r="F81" s="11" t="n">
-        <v>5.3</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="82" ht="14" customHeight="1">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>Haiyan Huang</t>
+          <t>Brian Corvese</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holding</t>
+          <t>Agenus</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -8286,22 +8286,22 @@
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>AGEN</t>
         </is>
       </c>
       <c r="F82" s="11" t="n">
-        <v>5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="83" ht="14" customHeight="1">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>Poh Kiong Tan</t>
+          <t>David Moradi</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holding</t>
+          <t>AudioEye</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -8316,22 +8316,22 @@
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>AEYE</t>
         </is>
       </c>
       <c r="F83" s="11" t="n">
-        <v>5</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="84" ht="14" customHeight="1">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>Soon Huat Lim</t>
+          <t>Tiago Miranda</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holding</t>
+          <t>Atlas Lithium</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -8346,22 +8346,22 @@
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>ATLX</t>
         </is>
       </c>
       <c r="F84" s="11" t="n">
-        <v>5</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Hock Goh</t>
+          <t>Charles Leykum</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Talon Capital (SPAC</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -8376,22 +8376,22 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>SKF-B.ST</t>
+          <t>TLNC</t>
         </is>
       </c>
       <c r="F85" s="11" t="n">
-        <v>4.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>Rebecca Grossman-Cohen</t>
+          <t>Paul Allen</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Airship AI Holdings</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -8406,22 +8406,22 @@
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>NYT</t>
+          <t>AISP</t>
         </is>
       </c>
       <c r="F86" s="11" t="n">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Michael Denham</t>
+          <t>David Allen</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>National Bank of Canada (Mon</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -8436,22 +8436,22 @@
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="F87" s="11" t="n">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>Nicholas Zangler</t>
+          <t>Laura Duda</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Viant Technology</t>
+          <t>The Goodyear Tire &amp; Rubber</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -8466,22 +8466,22 @@
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="F88" s="11" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="89" ht="14" customHeight="1">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Aris Kekedjian</t>
+          <t>Oscar Iglesias</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Stratasys (Printing Services</t>
+          <t>Codere Online Luxembourg</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -8496,22 +8496,22 @@
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>SSYS</t>
+          <t>CDROW</t>
         </is>
       </c>
       <c r="F89" s="11" t="n">
-        <v>3.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="90" ht="14" customHeight="1">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>Phillip Kardis</t>
+          <t>Martin Bork</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Chimera Investment</t>
+          <t>Navigator Holdings</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -8521,27 +8521,27 @@
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>CIM-PD</t>
+          <t>NVGS</t>
         </is>
       </c>
       <c r="F90" s="11" t="n">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="91" ht="14" customHeight="1">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>Subramaniam Viswanathan</t>
+          <t>Haiyan Huang</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Chimera Investment</t>
+          <t>Trident Digital Tech Holding</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -8551,27 +8551,27 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>CIM-PD</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="F91" s="11" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92" ht="14" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>Anelise Lara</t>
+          <t>Poh Kiong Tan</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>Trident Digital Tech Holding</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -8586,22 +8586,22 @@
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="F92" s="11" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>Josephine Linden</t>
+          <t>Soon Huat Lim</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Lands' End</t>
+          <t>Trident Digital Tech Holding</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -8611,27 +8611,27 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="F93" s="11" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>John McPherson</t>
+          <t>Hock Goh</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Commercial Metals</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8646,22 +8646,22 @@
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>SKF-B.ST</t>
         </is>
       </c>
       <c r="F94" s="11" t="n">
-        <v>2.9</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="95" ht="14" customHeight="1">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Richard Massey</t>
+          <t>Rebecca Grossman-Cohen</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Jena Acquisition II</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -8676,22 +8676,22 @@
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>JENA-UN</t>
+          <t>NYT</t>
         </is>
       </c>
       <c r="F95" s="11" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="96" ht="14" customHeight="1">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>John Campbell</t>
+          <t>Michael Denham</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Porch Group</t>
+          <t>National Bank of Canada (Mon</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8706,22 +8706,22 @@
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="F96" s="11" t="n">
-        <v>2.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Donald Dixon</t>
+          <t>Nicholas Zangler</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Amprius Technologies</t>
+          <t>Viant Technology</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8736,22 +8736,22 @@
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="F97" s="11" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>Sylvia Summers</t>
+          <t>Aris Kekedjian</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Stratasys (Printing Services</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8766,22 +8766,22 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>SSYS</t>
         </is>
       </c>
       <c r="F98" s="11" t="n">
-        <v>2.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>Phillip Kardis</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Chimera Investment</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8791,27 +8791,27 @@
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>CIM-PD</t>
         </is>
       </c>
       <c r="F99" s="11" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="100" ht="14" customHeight="1">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Alexander Krane</t>
+          <t>Subramaniam Viswanathan</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Chimera Investment</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8821,27 +8821,27 @@
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>CIM-PD</t>
         </is>
       </c>
       <c r="F100" s="11" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Andrea Pinarel</t>
+          <t>Anelise Lara</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
@@ -8856,22 +8856,22 @@
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="F101" s="11" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>David Kennedy</t>
+          <t>Josephine Linden</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Lands' End</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -8881,27 +8881,27 @@
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="F102" s="11" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="103" ht="14" customHeight="1">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Feyyaz Etiz</t>
+          <t>Sylvia Summers</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -8916,22 +8916,22 @@
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="F103" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Gustavo Baquero</t>
+          <t>John McPherson</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Commercial Metals</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
@@ -8946,22 +8946,22 @@
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="F104" s="11" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Linda Cook</t>
+          <t>Richard Massey</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Jena Acquisition II</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -8976,22 +8976,22 @@
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>JENA-UN</t>
         </is>
       </c>
       <c r="F105" s="11" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Michael Tuffin</t>
+          <t>John Campbell</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Porch Group</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -9006,22 +9006,22 @@
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="F106" s="11" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="107" ht="14" customHeight="1">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Nathan Mauzy</t>
+          <t>Donald Dixon</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Amprius Technologies</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -9036,11 +9036,11 @@
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>AMPX</t>
         </is>
       </c>
       <c r="F107" s="11" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1">
@@ -9166,12 +9166,12 @@
     <row r="112" ht="14" customHeight="1">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>Jane O'Keeffe</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Bancroft Fund</t>
+          <t>Woodside Energy Group</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -9186,7 +9186,7 @@
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>BCV-PA</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="F112" s="11" t="n">
@@ -9196,12 +9196,12 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>Jane O'Keeffe</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group</t>
+          <t>Bancroft Fund</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -9216,11 +9216,11 @@
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>BCV-PA</t>
         </is>
       </c>
       <c r="F113" s="11" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="114" ht="14" customHeight="1">

</xml_diff>

<commit_message>
Billionaire FO gap-fill + placeholder-CUSIP contamination fix
- Add 3 verified active 13F filers: Meritage Group (Nat Simons, $2.65B),
  Wildcat Capital (Bonderman FO), Thiel Macro (Peter Thiel); roster 455.
- Fix zero-CUSIP contamination: 000000000 (empty-filing placeholder) had
  been persisted as authority -> PRLD, painting 6 empty filings as phantom
  PRLD holders and mislabeling OrbiMed's $22M ImageneBio line as PRLD
  (double-count). Guards added in build_cusip_map (upsert validity),
  ingest_13f + ingest_13f_prior (skip zero rows, no authority lookup on
  placeholder CUSIPs), validate (I8d invariant). OrbiMed IMAGENEBIO -> IMA.
- PRLD smart_money_n 6.7 -> 2.7; IMA properly credited (OrbiMed top holder).
- Rescore + re-render all workbooks; validate 0 failures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzLWQfQoCmwwwE2QTFQZro
</commit_message>
<xml_diff>
--- a/people_monitor.xlsx
+++ b/people_monitor.xlsx
@@ -610,7 +610,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sourced from five PitchBook people-searches (1,984 individuals), each filtered to board/advisory roles.</t>
+          <t>Sourced from five PitchBook people-searches (1,983 individuals), each filtered to board/advisory roles.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="D5" s="11" t="n">
-        <v>13.3</v>
+        <v>17.3</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>4.3</v>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>1</v>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>1.6</v>
@@ -1273,7 +1273,7 @@
     <row r="11" ht="14" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>UAA</t>
+          <t>RIG</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -1283,26 +1283,26 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Under Armour, Inc.</t>
+          <t>Transocean Ltd.</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>38.3</v>
+        <v>32.4</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>1.8</v>
+        <v>4.8</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>2021</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Dawn Fitzpatrick</t>
+          <t>Margareth Ovrum</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -1312,14 +1312,14 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>RIG</t>
+          <t>HGV</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -1329,26 +1329,26 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Transocean Ltd.</t>
+          <t>Hilton Grand Vacations Inc</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>32.7</v>
+        <v>23.4</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="F12" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Margareth Ovrum</t>
+          <t>Leonard Potter</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
@@ -1358,14 +1358,14 @@
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>HGV</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -1375,26 +1375,26 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Hilton Grand Vacations Inc</t>
+          <t>Charter Communications, In</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>2011</t>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Leonard Potter</t>
+          <t>W. Conn</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
@@ -1404,14 +1404,14 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -1421,14 +1421,14 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Charter Communications, In</t>
+          <t>QXO, Inc.</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>19.7</v>
+        <v>17.5</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>5.7</v>
+        <v>7.4</v>
       </c>
       <c r="F14" s="12" t="n">
         <v>1</v>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>W. Conn</t>
+          <t>Mary Kissel</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1450,14 +1450,14 @@
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>TOL</t>
+          <t>MNRO</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -1467,26 +1467,26 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Toll Brothers, Inc.</t>
+          <t>Monro, Inc.</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>19.7</v>
+        <v>17.3</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="F15" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>2012</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Derek Kan</t>
+          <t>Hope Woodhouse</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -1503,7 +1503,7 @@
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>MNRO</t>
+          <t>SANA</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -1513,26 +1513,26 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Monro, Inc.</t>
+          <t>Sana Biotechnology, Inc.</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>17.4</v>
+        <v>16.6</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="F16" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>2012</t>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Hope Woodhouse</t>
+          <t>Richard Mulligan</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
@@ -1542,14 +1542,14 @@
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>SANA</t>
+          <t>UAA</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -1559,14 +1559,14 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Sana Biotechnology, Inc.</t>
+          <t>Under Armour, Inc.</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>16.6</v>
+        <v>14.9</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="F17" s="12" t="n">
         <v>1</v>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>Richard Mulligan</t>
+          <t>Dawn Fitzpatrick</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1588,14 +1588,14 @@
       </c>
       <c r="J17" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>TOL</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -1605,14 +1605,14 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>QXO, Inc.</t>
+          <t>Toll Brothers, Inc.</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>7.4</v>
+        <v>3.6</v>
       </c>
       <c r="F18" s="12" t="n">
         <v>1</v>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Mary Kissel</t>
+          <t>Derek Kan</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>COYA</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -1697,26 +1697,26 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>SandRidge Energy, Inc.</t>
+          <t>Coya Therapeutics, Inc.</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>2.6</v>
+        <v>1.1</v>
       </c>
       <c r="F20" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>1999</t>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Nancy Dunlap</t>
+          <t>Wilbur Ross</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
@@ -1726,14 +1726,14 @@
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1743,26 +1743,26 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Westrock Coffee Company</t>
+          <t>SandRidge Energy, Inc.</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>9.800000000000001</v>
+        <v>12.1</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
       <c r="F21" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>1999</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>Jeffrey Fox</t>
+          <t>Nancy Dunlap</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
@@ -1772,14 +1772,14 @@
       </c>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>Consumer Defensi</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -1789,14 +1789,14 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Coya Therapeutics, Inc.</t>
+          <t>Westrock Coffee Company</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="F22" s="12" t="n">
         <v>1</v>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>Wilbur Ross</t>
+          <t>Jeffrey Fox</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Defensi</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>PMTR</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -2019,14 +2019,14 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Perimeter Acquisition Corp</t>
+          <t>Lands' End, Inc.</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="E27" s="11" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="F27" s="12" t="n">
         <v>1</v>
@@ -2038,24 +2038,24 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Jack Selby</t>
+          <t>Josephine Linden</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>SKF-B.ST</t>
+          <t>PMTR</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -2065,14 +2065,14 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>AB SKF (publ)</t>
+          <t>Perimeter Acquisition Corp</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>4.9</v>
+        <v>5.3</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F28" s="12" t="n">
         <v>1</v>
@@ -2084,17 +2084,17 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Hock Goh</t>
+          <t>Jack Selby</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>4.9</v>
+        <v>5.2</v>
       </c>
       <c r="E29" s="11" t="n">
         <v>6.1</v>
@@ -2147,7 +2147,7 @@
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>SKF-B.ST</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Lands' End, Inc.</t>
+          <t>AB SKF (publ)</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="F30" s="12" t="n">
         <v>1</v>
@@ -2176,17 +2176,17 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>Josephine Linden</t>
+          <t>Hock Goh</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>CENX</t>
+          <t>OKLO</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -2295,36 +2295,36 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Century Aluminum Company</t>
+          <t>Oklo Inc.</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="E33" s="11" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="F33" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="10" t="inlineStr">
-        <is>
-          <t>1996</t>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>Andrew Michelmore</t>
+          <t>Samuel Altman</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E34" s="11" t="n">
         <v>1.7</v>
@@ -2377,7 +2377,7 @@
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>EVR</t>
+          <t>VIV</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -2387,14 +2387,14 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Evercore Inc.</t>
+          <t>Telefônica Brasil S.A.</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="F35" s="12" t="n">
         <v>1</v>
@@ -2406,24 +2406,24 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Knee</t>
+          <t>Peter Loscher</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>EVR</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
@@ -2433,14 +2433,14 @@
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Telefônica Brasil S.A.</t>
+          <t>Evercore Inc.</t>
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="E36" s="11" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F36" s="12" t="n">
         <v>1</v>
@@ -2452,17 +2452,17 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Peter Loscher</t>
+          <t>Jonathan Knee</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>OKLO</t>
+          <t>CENX</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -2709,36 +2709,36 @@
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Oklo Inc.</t>
+          <t>Century Aluminum Company</t>
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>-2.8</v>
+        <v>-3.6</v>
       </c>
       <c r="E42" s="11" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="F42" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>1996</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Samuel Altman</t>
+          <t>Andrew Michelmore</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
         </is>
       </c>
       <c r="D43" s="11" t="n">
-        <v>35.7</v>
+        <v>34.8</v>
       </c>
       <c r="E43" s="11" t="n">
         <v>1.9</v>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>28.3</v>
+        <v>29.3</v>
       </c>
       <c r="E44" s="11" t="n">
         <v>1.4</v>
@@ -2837,7 +2837,7 @@
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -2847,26 +2847,26 @@
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>H2O America</t>
+          <t>SLB N.V.</t>
         </is>
       </c>
       <c r="D45" s="11" t="n">
-        <v>20.7</v>
+        <v>19.9</v>
       </c>
       <c r="E45" s="11" t="n">
-        <v>0.9</v>
+        <v>9</v>
       </c>
       <c r="F45" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>2011</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
         <is>
-          <t>Gregory Landis</t>
+          <t>Tatiana Mitrova</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
@@ -2876,14 +2876,14 @@
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>HTO</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -2893,26 +2893,26 @@
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>SLB N.V.</t>
+          <t>H2O America</t>
         </is>
       </c>
       <c r="D46" s="11" t="n">
-        <v>19.3</v>
+        <v>19.6</v>
       </c>
       <c r="E46" s="11" t="n">
-        <v>9</v>
+        <v>0.9</v>
       </c>
       <c r="F46" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="10" t="inlineStr">
-        <is>
-          <t>2011</t>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>Tatiana Mitrova</t>
+          <t>Gregory Landis</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr">
@@ -2922,14 +2922,14 @@
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>XMTR</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -2939,14 +2939,14 @@
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>COMPASS Pathways plc</t>
+          <t>Xometry, Inc.</t>
         </is>
       </c>
       <c r="D47" s="11" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="E47" s="11" t="n">
-        <v>6.1</v>
+        <v>2.6</v>
       </c>
       <c r="F47" s="12" t="n">
         <v>1</v>
@@ -2958,24 +2958,24 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Annalisa Jenkins</t>
+          <t>Katharine Weymouth</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>FRPH</t>
+          <t>CMPS</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -2985,14 +2985,14 @@
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>FRP Holdings, Inc.</t>
+          <t>COMPASS Pathways plc</t>
         </is>
       </c>
       <c r="D48" s="11" t="n">
         <v>18.5</v>
       </c>
       <c r="E48" s="11" t="n">
-        <v>1.3</v>
+        <v>6.1</v>
       </c>
       <c r="F48" s="12" t="n">
         <v>1</v>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>John Baker</t>
+          <t>Annalisa Jenkins</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
@@ -3014,14 +3014,14 @@
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>XMTR</t>
+          <t>FRPH</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -3031,14 +3031,14 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Xometry, Inc.</t>
+          <t>FRP Holdings, Inc.</t>
         </is>
       </c>
       <c r="D49" s="11" t="n">
-        <v>18.1</v>
+        <v>18.5</v>
       </c>
       <c r="E49" s="11" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="F49" s="12" t="n">
         <v>1</v>
@@ -3050,17 +3050,17 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>Katharine Weymouth</t>
+          <t>John Baker</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>LNZA</t>
+          <t>ALLO</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
@@ -3307,26 +3307,26 @@
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>LanzaTech Global, Inc.</t>
+          <t>Allogene Therapeutics, Inc</t>
         </is>
       </c>
       <c r="D55" s="11" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="E55" s="11" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
       <c r="F55" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G55" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G55" s="10" t="inlineStr">
+        <is>
+          <t>2012</t>
         </is>
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>Thierry Pilenko</t>
+          <t>Franz Humer</t>
         </is>
       </c>
       <c r="I55" s="10" t="inlineStr">
@@ -3336,14 +3336,14 @@
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>UPWK</t>
+          <t>LNZA</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -3353,14 +3353,14 @@
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Upwork Inc.</t>
+          <t>LanzaTech Global, Inc.</t>
         </is>
       </c>
       <c r="D56" s="11" t="n">
-        <v>10.1</v>
+        <v>10.7</v>
       </c>
       <c r="E56" s="11" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="F56" s="12" t="n">
         <v>1</v>
@@ -3372,17 +3372,17 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>Glenn Kelman</t>
+          <t>Thierry Pilenko</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J56" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="D57" s="11" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="E57" s="11" t="n">
         <v>1.2</v>
@@ -3435,7 +3435,7 @@
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>ALLO</t>
+          <t>UPWK</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
@@ -3445,36 +3445,36 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Allogene Therapeutics, Inc</t>
+          <t>Upwork Inc.</t>
         </is>
       </c>
       <c r="D58" s="11" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="E58" s="11" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
       <c r="F58" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="10" t="inlineStr">
-        <is>
-          <t>2012</t>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>Franz Humer</t>
+          <t>Glenn Kelman</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
@@ -3583,14 +3583,14 @@
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>MP Materials Corp.</t>
+          <t>Semtech Corporation</t>
         </is>
       </c>
       <c r="D61" s="11" t="n">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
       <c r="E61" s="11" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="F61" s="12" t="n">
         <v>1</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>Randall Weisenburger</t>
+          <t>Sylvia Summers</t>
         </is>
       </c>
       <c r="I61" s="10" t="inlineStr">
@@ -3612,14 +3612,14 @@
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>ADAG</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -3629,14 +3629,14 @@
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Adagene Inc.</t>
+          <t>MP Materials Corp.</t>
         </is>
       </c>
       <c r="D62" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E62" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F62" s="12" t="n">
         <v>1</v>
@@ -3648,24 +3648,24 @@
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>Li Li</t>
+          <t>Randall Weisenburger</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>ADAG</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holdi</t>
+          <t>Adagene Inc.</t>
         </is>
       </c>
       <c r="D63" s="11" t="n">
@@ -3687,31 +3687,31 @@
       <c r="F63" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G63" s="10" t="inlineStr">
-        <is>
-          <t>2014</t>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>Poh Kiong Tan</t>
+          <t>Li Li</t>
         </is>
       </c>
       <c r="I63" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J63" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -3721,43 +3721,43 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Sierra Bancorp</t>
+          <t>Trident Digital Tech Holdi</t>
         </is>
       </c>
       <c r="D64" s="11" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="E64" s="11" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F64" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G64" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G64" s="10" t="inlineStr">
+        <is>
+          <t>2014</t>
         </is>
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>Laurence Dutto</t>
+          <t>Poh Kiong Tan</t>
         </is>
       </c>
       <c r="I64" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J64" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -3767,14 +3767,14 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>Semtech Corporation</t>
+          <t>Porch Group, Inc.</t>
         </is>
       </c>
       <c r="D65" s="11" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="E65" s="11" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="F65" s="12" t="n">
         <v>1</v>
@@ -3786,24 +3786,24 @@
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>Sylvia Summers</t>
+          <t>Amanda Reierson</t>
         </is>
       </c>
       <c r="I65" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J65" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -3813,14 +3813,14 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Porch Group, Inc.</t>
+          <t>Guardant Health, Inc.</t>
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
       <c r="F66" s="12" t="n">
         <v>1</v>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
-          <t>Amanda Reierson</t>
+          <t>Aaref Hilaly</t>
         </is>
       </c>
       <c r="I66" s="10" t="inlineStr">
@@ -3842,14 +3842,14 @@
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>BSRR</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -3859,14 +3859,14 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>TotalEnergies SE</t>
+          <t>Sierra Bancorp</t>
         </is>
       </c>
       <c r="D67" s="11" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="E67" s="11" t="n">
-        <v>3.2</v>
+        <v>0.1</v>
       </c>
       <c r="F67" s="12" t="n">
         <v>1</v>
@@ -3878,24 +3878,24 @@
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>Anelise Lara</t>
+          <t>Laurence Dutto</t>
         </is>
       </c>
       <c r="I67" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -3905,26 +3905,26 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Commercial Metals Company</t>
+          <t>TotalEnergies SE</t>
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="F68" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G68" s="10" t="inlineStr">
-        <is>
-          <t>2014</t>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>John McPherson</t>
+          <t>Anelise Lara</t>
         </is>
       </c>
       <c r="I68" s="10" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
         </is>
       </c>
       <c r="D69" s="11" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="E69" s="11" t="n">
         <v>0.8</v>
@@ -3987,7 +3987,7 @@
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
@@ -3997,26 +3997,26 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy plc</t>
+          <t>Commercial Metals Company</t>
         </is>
       </c>
       <c r="D70" s="11" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="E70" s="11" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="F70" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>John McPherson</t>
         </is>
       </c>
       <c r="I70" s="10" t="inlineStr">
@@ -4026,14 +4026,14 @@
       </c>
       <c r="J70" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>RLXXF</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
@@ -4043,26 +4043,26 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>RELX PLC</t>
+          <t>Harbour Energy plc</t>
         </is>
       </c>
       <c r="D71" s="11" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="E71" s="11" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="F71" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G71" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G71" s="10" t="inlineStr">
+        <is>
+          <t>2018</t>
         </is>
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>Suzanne Wood</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="I71" s="10" t="inlineStr">
@@ -4072,14 +4072,14 @@
       </c>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>UBSI</t>
+          <t>RLXXF</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
@@ -4089,43 +4089,43 @@
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>United Bankshares, Inc.</t>
+          <t>RELX PLC</t>
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G72" s="10" t="inlineStr">
-        <is>
-          <t>2003</t>
+        <v>1</v>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>J. Mcnamara,Michael Fitzgerald</t>
+          <t>Suzanne Wood</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>UBSI</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
@@ -4135,43 +4135,43 @@
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>Danaos Corporation</t>
+          <t>United Bankshares, Inc.</t>
         </is>
       </c>
       <c r="D73" s="11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E73" s="11" t="n">
         <v>1.4</v>
       </c>
-      <c r="E73" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F73" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73" s="10" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>Dimitris Vastarouchas</t>
+          <t>J. Mcnamara,Michael Fitzgerald</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
@@ -4181,43 +4181,43 @@
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group Ltd</t>
+          <t>Danaos Corporation</t>
         </is>
       </c>
       <c r="D74" s="11" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="E74" s="11" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F74" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G74" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2005</t>
         </is>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>Dimitris Vastarouchas</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J74" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>SFM</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
@@ -4227,14 +4227,14 @@
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>United Microelectronics Co</t>
+          <t>Sprouts Farmers Market, In</t>
         </is>
       </c>
       <c r="D75" s="11" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E75" s="11" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
       <c r="F75" s="12" t="n">
         <v>1</v>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
-          <t>Jason Wang</t>
+          <t>Douglas Rauch</t>
         </is>
       </c>
       <c r="I75" s="10" t="inlineStr">
@@ -4256,14 +4256,14 @@
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Defensi</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>EIPAF</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -4273,26 +4273,26 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Eni S.p.A.</t>
+          <t>Woodside Energy Group Ltd</t>
         </is>
       </c>
       <c r="D76" s="11" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="E76" s="11" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="F76" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G76" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>2022</t>
         </is>
       </c>
       <c r="H76" s="10" t="inlineStr">
         <is>
-          <t>Massimo Belcredi</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="I76" s="10" t="inlineStr">
@@ -4309,7 +4309,7 @@
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>SFM</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
@@ -4319,14 +4319,14 @@
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>Sprouts Farmers Market, In</t>
+          <t>United Microelectronics Co</t>
         </is>
       </c>
       <c r="D77" s="11" t="n">
-        <v>-0.9</v>
+        <v>0.8</v>
       </c>
       <c r="E77" s="11" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="F77" s="12" t="n">
         <v>1</v>
@@ -4338,7 +4338,7 @@
       </c>
       <c r="H77" s="10" t="inlineStr">
         <is>
-          <t>Douglas Rauch</t>
+          <t>Jason Wang</t>
         </is>
       </c>
       <c r="I77" s="10" t="inlineStr">
@@ -4348,14 +4348,14 @@
       </c>
       <c r="J77" s="10" t="inlineStr">
         <is>
-          <t>Consumer Defensi</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>EIPAF</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
@@ -4365,14 +4365,14 @@
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Guardant Health, Inc.</t>
+          <t>Eni S.p.A.</t>
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>-2.2</v>
+        <v>0.2</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>5.2</v>
+        <v>0.1</v>
       </c>
       <c r="F78" s="12" t="n">
         <v>1</v>
@@ -4384,17 +4384,17 @@
       </c>
       <c r="H78" s="10" t="inlineStr">
         <is>
-          <t>Aaref Hilaly</t>
+          <t>Massimo Belcredi</t>
         </is>
       </c>
       <c r="I78" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J78" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="D79" s="11" t="n">
-        <v>-6.2</v>
+        <v>-5.2</v>
       </c>
       <c r="E79" s="11" t="n">
         <v>1.3</v>
@@ -4541,66 +4541,66 @@
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Yoav Shaked</t>
+          <t>Keith Rabois</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Capital</t>
+          <t>tracked principal</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>DarioHealth</t>
+          <t>Affirm</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>DRIO</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>17</v>
+        <v>17.3</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>0.6</v>
+        <v>4.3</v>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Chairman &amp; Board Membe</t>
+          <t>Board Member</t>
         </is>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Keith Rabois</t>
+          <t>Yoav Shaked</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>tracked principal</t>
+          <t>Sequoia Capital</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Affirm</t>
+          <t>DarioHealth</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>DRIO</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>13.3</v>
+        <v>17</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>4.3</v>
+        <v>0.6</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Board Member</t>
+          <t>Chairman &amp; Board Membe</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4659,7 @@
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="F8" s="12" t="n">
         <v>1</v>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="F9" s="12" t="n">
         <v>1.6</v>
@@ -5625,12 +5625,12 @@
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Dawn Fitzpatrick</t>
+          <t>Margareth Ovrum</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Under Armour</t>
+          <t>Transocean</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -5645,22 +5645,22 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>UAA</t>
+          <t>RIG</t>
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>38.3</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Margareth Ovrum</t>
+          <t>Pamala Kaufman</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Transocean</t>
+          <t>Lindblad Expeditions Holding</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -5675,52 +5675,52 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>RIG</t>
+          <t>LIND</t>
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>32.7</v>
+        <v>29.3</v>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Pamala Kaufman</t>
+          <t>Viral Patel</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Lindblad Expeditions Holding</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Public Company</t>
+          <t>PE/Buyout</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="F7" s="12" t="n">
-        <v>28.3</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Ashok Srivastava</t>
+          <t>Leonard Potter</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Intuit</t>
+          <t>Hilton Grand Vacations</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -5735,52 +5735,52 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>HGV</t>
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>27.5</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Viral Patel</t>
+          <t>Ashok Srivastava</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Blackstone</t>
+          <t>Intuit</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>PE/Buyout</t>
+          <t>Public Company</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="F9" s="12" t="n">
-        <v>23.9</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Leonard Potter</t>
+          <t>Ashwini Kumar</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Hilton Grand Vacations</t>
+          <t>PayPal Holdings</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -5795,22 +5795,22 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>HGV</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Ashwini Kumar</t>
+          <t>W. Conn</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>PayPal Holdings</t>
+          <t>Charter Communications</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -5825,22 +5825,22 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>22.3</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Gregory Landis</t>
+          <t>Tatiana Mitrova</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>H2O America</t>
+          <t>SLB (Other Energy Services</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -5855,22 +5855,22 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>20.7</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>W. Conn</t>
+          <t>Gregory Landis</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Charter Communications</t>
+          <t>H2O America</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -5885,22 +5885,22 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>HTO</t>
         </is>
       </c>
       <c r="F13" s="12" t="n">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Derek Kan</t>
+          <t>Annalisa Jenkins</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Toll Brothers</t>
+          <t>COMPASS Pathways</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -5915,22 +5915,22 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>TOL</t>
+          <t>CMPS</t>
         </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>19.7</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Tatiana Mitrova</t>
+          <t>John Baker</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>SLB (Other Energy Services</t>
+          <t>FRP Holdings</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -5945,22 +5945,22 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>FRPH</t>
         </is>
       </c>
       <c r="F15" s="12" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Annalisa Jenkins</t>
+          <t>Andrew Crowley</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>COMPASS Pathways</t>
+          <t>Markel Group</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -5975,22 +5975,22 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>MKL</t>
         </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>John Baker</t>
+          <t>Brandon Lewis</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>FRP Holdings</t>
+          <t>Veon</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -6005,22 +6005,22 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>FRPH</t>
+          <t>VEON</t>
         </is>
       </c>
       <c r="F17" s="12" t="n">
-        <v>18.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Andrew Crowley</t>
+          <t>Duncan Perry</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Markel Group</t>
+          <t>Veon</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -6035,22 +6035,22 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>MKL</t>
+          <t>VEON</t>
         </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>18</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Brandon Lewis</t>
+          <t>Mary Kissel</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Veon</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -6065,22 +6065,22 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>VEON</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="F19" s="12" t="n">
-        <v>17.6</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Duncan Perry</t>
+          <t>Hope Woodhouse</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Veon</t>
+          <t>Monro</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -6095,22 +6095,22 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>VEON</t>
+          <t>MNRO</t>
         </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Hope Woodhouse</t>
+          <t>C. Wes Burton</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Monro</t>
+          <t>Vulcan Materials</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -6125,17 +6125,17 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>MNRO</t>
+          <t>VMC</t>
         </is>
       </c>
       <c r="F21" s="12" t="n">
-        <v>17.4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>C. Wes Burton</t>
+          <t>Cynthia Hostetler</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -6165,7 +6165,7 @@
     <row r="23" ht="14" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Cynthia Hostetler</t>
+          <t>David Clement</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -6195,7 +6195,7 @@
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>David Clement</t>
+          <t>Denson Franklin</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -6225,7 +6225,7 @@
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Denson Franklin</t>
+          <t>George Willis</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -6255,7 +6255,7 @@
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>George Willis</t>
+          <t>J. Hill</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -6285,7 +6285,7 @@
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>J. Hill</t>
+          <t>J. Thomas Hill</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -6315,7 +6315,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>J. Thomas Hill</t>
+          <t>Jerry Perkins</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -6345,7 +6345,7 @@
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Jerry Perkins</t>
+          <t>Mark Warren</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -6375,7 +6375,7 @@
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>Mark Warren</t>
+          <t>Mary Carlisle</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -6405,7 +6405,7 @@
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Mary Carlisle</t>
+          <t>Thomas Fanning</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -6435,12 +6435,12 @@
     <row r="32" ht="14" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Thomas Fanning</t>
+          <t>Richard Mulligan</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Vulcan Materials</t>
+          <t>Sana Biotechnology</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -6455,22 +6455,22 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>VMC</t>
+          <t>SANA</t>
         </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>17</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Richard Mulligan</t>
+          <t>Danny Shepherd</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Sana Biotechnology</t>
+          <t>Beazer Homes USA</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -6485,22 +6485,22 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>SANA</t>
+          <t>BZH</t>
         </is>
       </c>
       <c r="F33" s="12" t="n">
-        <v>16.6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>David Wright</t>
+          <t>Michael Insulan</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Rezolve Ai</t>
+          <t>Electra Battery Materials</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -6510,27 +6510,27 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>RZLVW</t>
+          <t>ELBM</t>
         </is>
       </c>
       <c r="F34" s="12" t="n">
-        <v>16.4</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Danny Shepherd</t>
+          <t>David Wright</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Beazer Homes USA</t>
+          <t>Rezolve Ai</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -6540,27 +6540,27 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>BZH</t>
+          <t>RZLVW</t>
         </is>
       </c>
       <c r="F35" s="12" t="n">
-        <v>16</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Michael Insulan</t>
+          <t>Richard Russell</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Electra Battery Materials</t>
+          <t>LM Funding America</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -6575,22 +6575,22 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>ELBM</t>
+          <t>LMFA</t>
         </is>
       </c>
       <c r="F36" s="12" t="n">
-        <v>15.9</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Kenneth Gunderman</t>
+          <t>Dawn Fitzpatrick</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Uniti Group (Financial Servi</t>
+          <t>Under Armour</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -6605,22 +6605,22 @@
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>UAA</t>
         </is>
       </c>
       <c r="F37" s="12" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Richard Russell</t>
+          <t>Derek Kan</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>LM Funding America</t>
+          <t>Toll Brothers</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -6635,22 +6635,22 @@
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>LMFA</t>
+          <t>TOL</t>
         </is>
       </c>
       <c r="F38" s="12" t="n">
-        <v>15.1</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Mary Kissel</t>
+          <t>Meryl Hartzband</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>Everest Group (Hamilton</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -6665,22 +6665,22 @@
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="F39" s="12" t="n">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Meryl Hartzband</t>
+          <t>Jonathan Christodoro</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Everest Group (Hamilton</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -6695,17 +6695,17 @@
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>XRXDW</t>
         </is>
       </c>
       <c r="F40" s="12" t="n">
-        <v>13.5</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Christodoro</t>
+          <t>Louis Pastor</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -6735,12 +6735,12 @@
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Louis Pastor</t>
+          <t>Joseph Flaim</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Iamgold</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -6750,27 +6750,27 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>XRXDW</t>
+          <t>IAG</t>
         </is>
       </c>
       <c r="F42" s="12" t="n">
-        <v>13.2</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Joseph Flaim</t>
+          <t>Wilbur Ross</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Iamgold</t>
+          <t>Coya Therapeutics</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -6780,27 +6780,27 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>IAG</t>
+          <t>COYA</t>
         </is>
       </c>
       <c r="F43" s="12" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>James Nelson</t>
+          <t>Franz Humer</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Global Net Lease</t>
+          <t>Allogene Therapeutics</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -6815,22 +6815,22 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>GNL</t>
+          <t>ALLO</t>
         </is>
       </c>
       <c r="F44" s="12" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Frates</t>
+          <t>James Nelson</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>SandRidge Energy</t>
+          <t>Global Net Lease</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -6845,17 +6845,17 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>GNL</t>
         </is>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.1</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>Nancy Dunlap</t>
+          <t>Jonathan Frates</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -6885,12 +6885,12 @@
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Thierry Pilenko</t>
+          <t>Nancy Dunlap</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>LanzaTech Global</t>
+          <t>SandRidge Energy</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -6905,11 +6905,11 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>LNZA</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F47" s="12" t="n">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
@@ -6939,18 +6939,18 @@
         </is>
       </c>
       <c r="F48" s="12" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Sandra Bell</t>
+          <t>Kathleen Quirk</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Dye &amp; Durham</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -6960,27 +6960,27 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>DYNDF</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="F49" s="12" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Kelly Osborne</t>
+          <t>Thierry Pilenko</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Kinross Gold</t>
+          <t>LanzaTech Global</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -6995,22 +6995,22 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>KGCRF</t>
+          <t>LNZA</t>
         </is>
       </c>
       <c r="F50" s="12" t="n">
-        <v>10.4</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>Stephen Gunther</t>
+          <t>Sandra Bell</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Shoulder Innovations</t>
+          <t>Dye &amp; Durham</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -7025,22 +7025,22 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>DYNDF</t>
         </is>
       </c>
       <c r="F51" s="12" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Anthony Williams</t>
+          <t>Stephen Gunther</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Akamai Technologies</t>
+          <t>Shoulder Innovations</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -7050,16 +7050,16 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>AKAM</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F52" s="12" t="n">
-        <v>10.1</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
@@ -7089,18 +7089,18 @@
         </is>
       </c>
       <c r="F53" s="12" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>Franz Humer</t>
+          <t>Kelly Osborne</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Allogene Therapeutics</t>
+          <t>Kinross Gold</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -7115,22 +7115,22 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>ALLO</t>
+          <t>KGCRF</t>
         </is>
       </c>
       <c r="F54" s="12" t="n">
-        <v>10</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Jeffrey Fox</t>
+          <t>Anthony Williams</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Westrock Coffee</t>
+          <t>Akamai Technologies</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -7145,22 +7145,22 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>AKAM</t>
         </is>
       </c>
       <c r="F55" s="12" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Wilbur Ross</t>
+          <t>Kenneth Gunderman</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Coya Therapeutics</t>
+          <t>Uniti Group (Financial Servi</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -7175,22 +7175,22 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="F56" s="12" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Wendy Teramoto</t>
+          <t>Jeffrey Fox</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>The Greenbrier Companies</t>
+          <t>Westrock Coffee</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -7205,22 +7205,22 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>GBX</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="F57" s="12" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>R. Cox</t>
+          <t>Wendy Teramoto</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Terex</t>
+          <t>The Greenbrier Companies</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -7235,22 +7235,22 @@
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>GBX</t>
         </is>
       </c>
       <c r="F58" s="12" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Kathleen Quirk</t>
+          <t>Allan D. Schoening</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Civeo</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -7265,11 +7265,11 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>CVEO</t>
         </is>
       </c>
       <c r="F59" s="12" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
@@ -7299,78 +7299,78 @@
         </is>
       </c>
       <c r="F60" s="12" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Allan D. Schoening</t>
+          <t>Dominic Picone</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Civeo</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Public Company</t>
+          <t>PE/Buyout</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>CVEO</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="F61" s="12" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Dominic Picone</t>
+          <t>Daniel Sansone</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>Ingevity</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>PE/Buyout</t>
+          <t>Public Company</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>NGVT</t>
         </is>
       </c>
       <c r="F62" s="12" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Daniel Sansone</t>
+          <t>David Habachy</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Ingevity</t>
+          <t>Ring Energy</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -7385,22 +7385,22 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>NGVT</t>
+          <t>REI</t>
         </is>
       </c>
       <c r="F63" s="12" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>David Habachy</t>
+          <t>Pam Kaufman</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Ring Energy</t>
+          <t>Paramount Skydance</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -7415,22 +7415,22 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>REI</t>
+          <t>PSKY</t>
         </is>
       </c>
       <c r="F64" s="12" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Pam Kaufman</t>
+          <t>Len Blavatnik</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Paramount Skydance</t>
+          <t>Warner Music Group</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>PSKY</t>
+          <t>WMG</t>
         </is>
       </c>
       <c r="F65" s="12" t="n">
@@ -7455,12 +7455,12 @@
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Len Blavatnik</t>
+          <t>Randle Reece</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Warner Music Group</t>
+          <t>AMN Healthcare Services</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -7475,22 +7475,22 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>WMG</t>
+          <t>AMN</t>
         </is>
       </c>
       <c r="F66" s="12" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Randle Reece</t>
+          <t>Mark DiPaolo</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>AMN Healthcare Services</t>
+          <t>Innoviva</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -7505,22 +7505,22 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>AMN</t>
+          <t>INVA</t>
         </is>
       </c>
       <c r="F67" s="12" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>Mark DiPaolo</t>
+          <t>Tim Cahill</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Innoviva</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -7535,7 +7535,7 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="F68" s="12" t="n">
@@ -7545,12 +7545,12 @@
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Tim Cahill</t>
+          <t>Robert Colligan</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Lockheed Martin</t>
+          <t>Dynex Capital</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -7560,12 +7560,12 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>DX</t>
         </is>
       </c>
       <c r="F69" s="12" t="n">
@@ -7575,12 +7575,12 @@
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>Robert Colligan</t>
+          <t>David Allen</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Dynex Capital</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -7590,16 +7590,16 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="F70" s="12" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
@@ -7635,12 +7635,12 @@
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>David Moradi</t>
+          <t>Sylvia Summers</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>AudioEye</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="F72" s="12" t="n">
@@ -7665,12 +7665,12 @@
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>Tiago Miranda</t>
+          <t>David Moradi</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Atlas Lithium</t>
+          <t>AudioEye</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -7685,22 +7685,22 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>ATLX</t>
+          <t>AEYE</t>
         </is>
       </c>
       <c r="F73" s="12" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>Charles Leykum</t>
+          <t>Tiago Miranda</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Talon Capital (SPAC</t>
+          <t>Atlas Lithium</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -7715,22 +7715,22 @@
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>TLNC</t>
+          <t>ATLX</t>
         </is>
       </c>
       <c r="F74" s="12" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>David Allen</t>
+          <t>Randall Weisenburger</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -7745,22 +7745,22 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="F75" s="12" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Tony Buffin</t>
+          <t>Charles Leykum</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>DFS Furniture</t>
+          <t>Talon Capital (SPAC</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -7775,22 +7775,22 @@
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>DFS.L</t>
+          <t>TLNC</t>
         </is>
       </c>
       <c r="F76" s="12" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>Paul Allen</t>
+          <t>Tony Buffin</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Airship AI Holdings</t>
+          <t>DFS Furniture</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -7805,22 +7805,22 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>DFS.L</t>
         </is>
       </c>
       <c r="F77" s="12" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>Randall Weisenburger</t>
+          <t>Paul Allen</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>MP Materials</t>
+          <t>Airship AI Holdings</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>AISP</t>
         </is>
       </c>
       <c r="F78" s="12" t="n">
@@ -7845,12 +7845,12 @@
     <row r="79" ht="14" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>Martin Bork</t>
+          <t>Josephine Linden</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Navigator Holdings</t>
+          <t>Lands' End</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -7860,27 +7860,27 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>NVGS</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="F79" s="12" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>Laura Duda</t>
+          <t>Martin Bork</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>The Goodyear Tire &amp; Rubber</t>
+          <t>Navigator Holdings</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -7895,22 +7895,22 @@
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>NVGS</t>
         </is>
       </c>
       <c r="F80" s="12" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Oscar Iglesias</t>
+          <t>Laura Duda</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Codere Online Luxembourg</t>
+          <t>The Goodyear Tire &amp; Rubber</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>CDROW</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="F81" s="12" t="n">
@@ -7935,12 +7935,12 @@
     <row r="82" ht="14" customHeight="1">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>Haiyan Huang</t>
+          <t>Oscar Iglesias</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holding</t>
+          <t>Codere Online Luxembourg</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -7955,22 +7955,22 @@
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>CDROW</t>
         </is>
       </c>
       <c r="F82" s="12" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="83" ht="14" customHeight="1">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>Poh Kiong Tan</t>
+          <t>Rebecca Grossman-Cohen</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Trident Digital Tech Holding</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>TDTH</t>
+          <t>NYT</t>
         </is>
       </c>
       <c r="F83" s="12" t="n">
@@ -7995,7 +7995,7 @@
     <row r="84" ht="14" customHeight="1">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>Soon Huat Lim</t>
+          <t>Haiyan Huang</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
@@ -8025,12 +8025,12 @@
     <row r="85" ht="14" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Rebecca Grossman-Cohen</t>
+          <t>Poh Kiong Tan</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Trident Digital Tech Holding</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -8045,7 +8045,7 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>NYT</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="F85" s="12" t="n">
@@ -8055,12 +8055,12 @@
     <row r="86" ht="14" customHeight="1">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>Hock Goh</t>
+          <t>Soon Huat Lim</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>SKF</t>
+          <t>Trident Digital Tech Holding</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -8075,22 +8075,22 @@
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>SKF-B.ST</t>
+          <t>TDTH</t>
         </is>
       </c>
       <c r="F86" s="12" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Michael Denham</t>
+          <t>Hock Goh</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>National Bank of Canada (Mon</t>
+          <t>SKF</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -8105,22 +8105,22 @@
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>SKF-B.ST</t>
         </is>
       </c>
       <c r="F87" s="12" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>Josephine Linden</t>
+          <t>R. Cox</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Lands' End</t>
+          <t>Terex</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -8130,27 +8130,27 @@
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="F88" s="12" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="89" ht="14" customHeight="1">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Nicholas Zangler</t>
+          <t>Michael Denham</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Viant Technology</t>
+          <t>National Bank of Canada (Mon</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -8165,22 +8165,22 @@
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="F89" s="12" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="90" ht="14" customHeight="1">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>Aris Kekedjian</t>
+          <t>John Campbell</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Stratasys (Printing Services</t>
+          <t>Porch Group</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -8195,22 +8195,22 @@
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>SSYS</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="F90" s="12" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="91" ht="14" customHeight="1">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>Phillip Kardis</t>
+          <t>Nicholas Zangler</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Chimera Investment</t>
+          <t>Viant Technology</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -8220,27 +8220,27 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>CIM-PD</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="F91" s="12" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="92" ht="14" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>Subramaniam Viswanathan</t>
+          <t>Aris Kekedjian</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Chimera Investment</t>
+          <t>Stratasys (Printing Services</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -8250,27 +8250,27 @@
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>CIM-PD</t>
+          <t>SSYS</t>
         </is>
       </c>
       <c r="F92" s="12" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>Sylvia Summers</t>
+          <t>Phillip Kardis</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Chimera Investment</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -8280,27 +8280,27 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>CIM-PD</t>
         </is>
       </c>
       <c r="F93" s="12" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>John Campbell</t>
+          <t>Subramaniam Viswanathan</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Porch Group</t>
+          <t>Chimera Investment</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8310,16 +8310,16 @@
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>CIM-PD</t>
         </is>
       </c>
       <c r="F94" s="12" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="95" ht="14" customHeight="1">
@@ -8355,12 +8355,12 @@
     <row r="96" ht="14" customHeight="1">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>John McPherson</t>
+          <t>Donald Dixon</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Commercial Metals</t>
+          <t>Amprius Technologies</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8375,22 +8375,22 @@
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>AMPX</t>
         </is>
       </c>
       <c r="F96" s="12" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Richard Massey</t>
+          <t>John McPherson</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Jena Acquisition II</t>
+          <t>Commercial Metals</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8405,22 +8405,22 @@
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>JENA-UN</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="F97" s="12" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>Donald Dixon</t>
+          <t>Richard Massey</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Amprius Technologies</t>
+          <t>Jena Acquisition II</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8435,22 +8435,22 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>JENA-UN</t>
         </is>
       </c>
       <c r="F98" s="12" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>Michael Dougherty</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Polaris (Automotive</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -8465,22 +8465,22 @@
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>PII</t>
         </is>
       </c>
       <c r="F99" s="12" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="100" ht="14" customHeight="1">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Alexander Krane</t>
+          <t>Chris Siu</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>Aehr Test Systems</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
@@ -8495,17 +8495,17 @@
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="F100" s="12" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Andrea Pinarel</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
@@ -8535,7 +8535,7 @@
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>David Kennedy</t>
+          <t>Alexander Krane</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
@@ -8565,7 +8565,7 @@
     <row r="103" ht="14" customHeight="1">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Feyyaz Etiz</t>
+          <t>Andrea Pinarel</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
@@ -8595,7 +8595,7 @@
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Gustavo Baquero</t>
+          <t>David Kennedy</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
@@ -8625,7 +8625,7 @@
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Linda Cook</t>
+          <t>Feyyaz Etiz</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
@@ -8655,7 +8655,7 @@
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Michael Tuffin</t>
+          <t>Gustavo Baquero</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
@@ -8685,7 +8685,7 @@
     <row r="107" ht="14" customHeight="1">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Nathan Mauzy</t>
+          <t>Linda Cook</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
@@ -8715,12 +8715,12 @@
     <row r="108" ht="14" customHeight="1">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>Suzanne Wood</t>
+          <t>Michael Tuffin</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>RELX (Information Technology</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -8735,22 +8735,22 @@
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>RLXXF</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F108" s="12" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" ht="14" customHeight="1">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>Michael Dougherty</t>
+          <t>Nathan Mauzy</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>Polaris (Automotive</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -8765,22 +8765,22 @@
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>PII</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F109" s="12" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" ht="14" customHeight="1">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>Chris Siu</t>
+          <t>Suzanne Wood</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Aehr Test Systems</t>
+          <t>RELX (Information Technology</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -8795,22 +8795,22 @@
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>RLXXF</t>
         </is>
       </c>
       <c r="F110" s="12" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>Dimitris Vastarouchas</t>
+          <t>Raffaele Zagari</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Danaos</t>
+          <t>Star Bulk Carriers</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -8820,27 +8820,27 @@
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="F111" s="12" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="112" ht="14" customHeight="1">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>Andrew Michelmore</t>
+          <t>Dimitris Vastarouchas</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Century Aluminum</t>
+          <t>Danaos</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -8850,12 +8850,12 @@
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>CENX</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="F112" s="12" t="n">
@@ -8865,12 +8865,12 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>Raffaele Zagari</t>
+          <t>Douglas Rauch</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>Star Bulk Carriers</t>
+          <t>Sprouts Farmers Market</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>SFM</t>
         </is>
       </c>
       <c r="F113" s="12" t="n">
@@ -8895,12 +8895,12 @@
     <row r="114" ht="14" customHeight="1">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>Peter Loscher</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t>Telefónica</t>
+          <t>Woodside Energy Group</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="F114" s="12" t="n">
@@ -8925,12 +8925,12 @@
     <row r="115" ht="14" customHeight="1">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>Peter Loscher</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group</t>
+          <t>Telefónica</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>VIV</t>
         </is>
       </c>
       <c r="F115" s="12" t="n">
@@ -9195,12 +9195,12 @@
     <row r="124" ht="14" customHeight="1">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>Douglas Rauch</t>
+          <t>Kent Yee</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>Sprouts Farmers Market</t>
+          <t>DXP Enterprises</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
@@ -9215,22 +9215,22 @@
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>SFM</t>
+          <t>DXPE</t>
         </is>
       </c>
       <c r="F124" s="12" t="n">
-        <v>-0.9</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="125" ht="14" customHeight="1">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>Kent Yee</t>
+          <t>Andrew Michelmore</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>DXP Enterprises</t>
+          <t>Century Aluminum</t>
         </is>
       </c>
       <c r="C125" s="10" t="inlineStr">
@@ -9245,11 +9245,11 @@
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>DXPE</t>
+          <t>CENX</t>
         </is>
       </c>
       <c r="F125" s="12" t="n">
-        <v>-1.1</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="126" ht="14" customHeight="1">
@@ -9279,7 +9279,7 @@
         </is>
       </c>
       <c r="F126" s="12" t="n">
-        <v>-6.2</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="127" ht="14" customHeight="1">

</xml_diff>

<commit_message>
Wire latent-swap/Form144/N-PORT into radar + render 3 new sheets
- Broker Swap Radar: disclosed-swap cross-reference (PENN/HG Vora fires the
  1.6x multiplier) + Form 144 contra column (WBI: UBS building vs $254M/4
  filers proposing to sell). PENN = disclosed swap AND desk spike.
- Latent Ownership sheet: 269 13Ds with hidden warrants/converts/blockers/
  board rights/swaps (TLPH 6-feature, FATE 14.99% blocker + UBS swap).
- N-PORT Monthly sheet: marquee funds' monthly holdings incl. foreign/private
  names 13F omits (Baron's $1.6B SpaceX, Sequoia's Rolls-Royce, Davis Samsung).
- 10 new compounders scored; roster 479. validate 0 failures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzLWQfQoCmwwwE2QTFQZro
</commit_message>
<xml_diff>
--- a/people_monitor.xlsx
+++ b/people_monitor.xlsx
@@ -1011,10 +1011,10 @@
         </is>
       </c>
       <c r="D5" s="11" t="n">
-        <v>18.8</v>
+        <v>19.3</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>4.4</v>
+        <v>5.7</v>
       </c>
       <c r="F5" s="12" t="n">
         <v>1</v>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0.9</v>
@@ -1287,10 +1287,10 @@
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>1</v>
@@ -1471,10 +1471,10 @@
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>18.3</v>
+        <v>18.6</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="F15" s="12" t="n">
         <v>1</v>
@@ -1517,10 +1517,10 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>16.7</v>
+        <v>16.9</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="F16" s="12" t="n">
         <v>1</v>
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>14.5</v>
+        <v>15.3</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="F18" s="12" t="n">
         <v>1</v>
@@ -1917,7 +1917,7 @@
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -1927,14 +1927,14 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Innoviva, Inc.</t>
+          <t>ConocoPhillips</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
       <c r="E25" s="11" t="n">
-        <v>1.6</v>
+        <v>7.2</v>
       </c>
       <c r="F25" s="12" t="n">
         <v>1</v>
@@ -1946,24 +1946,24 @@
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t>Mark DiPaolo</t>
+          <t>Sharmila Mulligan</t>
         </is>
       </c>
       <c r="I25" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>DFS.L</t>
+          <t>INVA</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -1973,14 +1973,14 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>DFS Furniture plc</t>
+          <t>Innoviva, Inc.</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
       <c r="E26" s="11" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="F26" s="12" t="n">
         <v>1</v>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Tony Buffin</t>
+          <t>Mark DiPaolo</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
@@ -2002,14 +2002,14 @@
       </c>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>DFS.L</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -2019,14 +2019,14 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Lands' End, Inc.</t>
+          <t>DFS Furniture plc</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="E27" s="11" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="F27" s="12" t="n">
         <v>1</v>
@@ -2038,12 +2038,12 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Josephine Linden</t>
+          <t>Tony Buffin</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J27" s="10" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>PMTR</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -2065,11 +2065,11 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Perimeter Acquisition Corp</t>
+          <t>Lands' End, Inc.</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="E28" s="11" t="n">
         <v>1.9</v>
@@ -2084,24 +2084,24 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Jack Selby</t>
+          <t>Josephine Linden</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>PMTR</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -2111,14 +2111,14 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>ConocoPhillips</t>
+          <t>Perimeter Acquisition Corp</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>5.2</v>
+        <v>1.9</v>
       </c>
       <c r="F29" s="12" t="n">
         <v>1</v>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>Sharmila Mulligan</t>
+          <t>Jack Selby</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>OKLO</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -2295,14 +2295,14 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Oklo Inc.</t>
+          <t>Star Bulk Carriers Corp.</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="E33" s="11" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="F33" s="12" t="n">
         <v>1</v>
@@ -2314,24 +2314,24 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>Samuel Altman</t>
+          <t>Raffaele Zagari</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Titans &amp; Concentrated Ma</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>OKLO</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -2341,14 +2341,14 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Star Bulk Carriers Corp.</t>
+          <t>Oklo Inc.</t>
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="E34" s="11" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>1</v>
@@ -2360,24 +2360,24 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>Raffaele Zagari</t>
+          <t>Samuel Altman</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Titans &amp; Concentrated Ma</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>EVR</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -2387,14 +2387,14 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Telefônica Brasil S.A.</t>
+          <t>Evercore Inc.</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
         <v>1.1</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="F35" s="12" t="n">
         <v>1</v>
@@ -2406,24 +2406,24 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>Peter Loscher</t>
+          <t>Jonathan Knee</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>EVR</t>
+          <t>VIV</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
@@ -2433,14 +2433,14 @@
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Evercore Inc.</t>
+          <t>Telefônica Brasil S.A.</t>
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="E36" s="11" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="F36" s="12" t="n">
         <v>1</v>
@@ -2452,17 +2452,17 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Knee</t>
+          <t>Peter Loscher</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
         </is>
       </c>
       <c r="D45" s="11" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
       <c r="E45" s="11" t="n">
         <v>1.5</v>
@@ -2943,10 +2943,10 @@
         </is>
       </c>
       <c r="D47" s="11" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="E47" s="11" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F47" s="12" t="n">
         <v>3</v>
@@ -2992,7 +2992,7 @@
         <v>18.7</v>
       </c>
       <c r="E48" s="11" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="F48" s="12" t="n">
         <v>1</v>
@@ -3021,7 +3021,7 @@
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>FRPH</t>
+          <t>XMTR</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -3031,14 +3031,14 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>FRP Holdings, Inc.</t>
+          <t>Xometry, Inc.</t>
         </is>
       </c>
       <c r="D49" s="11" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="E49" s="11" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="F49" s="12" t="n">
         <v>1</v>
@@ -3050,24 +3050,24 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>John Baker</t>
+          <t>Katharine Weymouth</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>FRPH</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -3077,14 +3077,14 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>COMPASS Pathways plc</t>
+          <t>FRP Holdings, Inc.</t>
         </is>
       </c>
       <c r="D50" s="11" t="n">
         <v>18.5</v>
       </c>
       <c r="E50" s="11" t="n">
-        <v>6.1</v>
+        <v>1.3</v>
       </c>
       <c r="F50" s="12" t="n">
         <v>1</v>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>Annalisa Jenkins</t>
+          <t>John Baker</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -3106,14 +3106,14 @@
       </c>
       <c r="J50" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>XMTR</t>
+          <t>VEON</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -3123,43 +3123,43 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Xometry, Inc.</t>
+          <t>VEON Ltd.</t>
         </is>
       </c>
       <c r="D51" s="11" t="n">
-        <v>18.5</v>
+        <v>17.6</v>
       </c>
       <c r="E51" s="11" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>2</v>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>2023</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Katharine Weymouth</t>
+          <t>Brandon Lewis,Duncan Perry</t>
         </is>
       </c>
       <c r="I51" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J51" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Se</t>
         </is>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>VEON</t>
+          <t>DRIO</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -3169,43 +3169,43 @@
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>VEON Ltd.</t>
+          <t>DarioHealth Corp.</t>
         </is>
       </c>
       <c r="D52" s="11" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="E52" s="11" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>2023</t>
+        <v>1</v>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Brandon Lewis,Duncan Perry</t>
+          <t>Yoav Shaked</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>Communication Se</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>DRIO</t>
+          <t>BZH</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
@@ -3215,14 +3215,14 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>DarioHealth Corp.</t>
+          <t>Beazer Homes USA, Inc.</t>
         </is>
       </c>
       <c r="D53" s="11" t="n">
-        <v>17.4</v>
+        <v>16.1</v>
       </c>
       <c r="E53" s="11" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="F53" s="12" t="n">
         <v>1</v>
@@ -3234,24 +3234,24 @@
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>Yoav Shaked</t>
+          <t>Danny Shepherd</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Cyclica</t>
         </is>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>BZH</t>
+          <t>CMPS</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
@@ -3261,14 +3261,14 @@
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Beazer Homes USA, Inc.</t>
+          <t>COMPASS Pathways plc</t>
         </is>
       </c>
       <c r="D54" s="11" t="n">
-        <v>16.1</v>
+        <v>13.5</v>
       </c>
       <c r="E54" s="11" t="n">
-        <v>2.1</v>
+        <v>6.2</v>
       </c>
       <c r="F54" s="12" t="n">
         <v>1</v>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>Danny Shepherd</t>
+          <t>Annalisa Jenkins</t>
         </is>
       </c>
       <c r="I54" s="10" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclica</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="D57" s="11" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="E57" s="11" t="n">
         <v>2.5</v>
@@ -3587,10 +3587,10 @@
         </is>
       </c>
       <c r="D61" s="11" t="n">
-        <v>6.6</v>
+        <v>7.3</v>
       </c>
       <c r="E61" s="11" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="F61" s="12" t="n">
         <v>1</v>
@@ -3679,10 +3679,10 @@
         </is>
       </c>
       <c r="D63" s="11" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="E63" s="11" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="F63" s="12" t="n">
         <v>1</v>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="D65" s="11" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="E65" s="11" t="n">
         <v>1.3</v>
@@ -3803,7 +3803,7 @@
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -3813,14 +3813,14 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Sierra Bancorp</t>
+          <t>Guardant Health, Inc.</t>
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>0.1</v>
+        <v>4.9</v>
       </c>
       <c r="F66" s="12" t="n">
         <v>1</v>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="H66" s="10" t="inlineStr">
         <is>
-          <t>Laurence Dutto</t>
+          <t>Aaref Hilaly</t>
         </is>
       </c>
       <c r="I66" s="10" t="inlineStr">
@@ -3842,14 +3842,14 @@
       </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Healthcare</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>BSRR</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -3859,43 +3859,43 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Commercial Metals Company</t>
+          <t>Sierra Bancorp</t>
         </is>
       </c>
       <c r="D67" s="11" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="E67" s="11" t="n">
-        <v>1.8</v>
+        <v>0.1</v>
       </c>
       <c r="F67" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G67" s="10" t="inlineStr">
-        <is>
-          <t>2014</t>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>John McPherson</t>
+          <t>Laurence Dutto</t>
         </is>
       </c>
       <c r="I67" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J67" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -3905,43 +3905,43 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Guardant Health, Inc.</t>
+          <t>Commercial Metals Company</t>
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>4.3</v>
+        <v>1.9</v>
       </c>
       <c r="F68" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G68" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>2014</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Aaref Hilaly</t>
+          <t>John McPherson</t>
         </is>
       </c>
       <c r="I68" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J68" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
@@ -3951,14 +3951,14 @@
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Amprius Technologies, Inc.</t>
+          <t>TotalEnergies SE</t>
         </is>
       </c>
       <c r="D69" s="11" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="E69" s="11" t="n">
-        <v>0.8</v>
+        <v>3.6</v>
       </c>
       <c r="F69" s="12" t="n">
         <v>1</v>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="H69" s="10" t="inlineStr">
         <is>
-          <t>Donald Dixon</t>
+          <t>Anelise Lara</t>
         </is>
       </c>
       <c r="I69" s="10" t="inlineStr">
@@ -3980,14 +3980,14 @@
       </c>
       <c r="J69" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>AMPX</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
@@ -3997,14 +3997,14 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>TotalEnergies SE</t>
+          <t>Amprius Technologies, Inc.</t>
         </is>
       </c>
       <c r="D70" s="11" t="n">
         <v>3.3</v>
       </c>
       <c r="E70" s="11" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="F70" s="12" t="n">
         <v>1</v>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>Anelise Lara</t>
+          <t>Donald Dixon</t>
         </is>
       </c>
       <c r="I70" s="10" t="inlineStr">
@@ -4026,14 +4026,14 @@
       </c>
       <c r="J70" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>RLXXF</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
@@ -4043,26 +4043,26 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy plc</t>
+          <t>RELX PLC</t>
         </is>
       </c>
       <c r="D71" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E71" s="11" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="F71" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G71" s="10" t="inlineStr">
-        <is>
-          <t>2018</t>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>Suzanne Wood</t>
         </is>
       </c>
       <c r="I71" s="10" t="inlineStr">
@@ -4072,14 +4072,14 @@
       </c>
       <c r="J71" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>SFM</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
@@ -4089,26 +4089,26 @@
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Sprouts Farmers Market, In</t>
+          <t>Harbour Energy plc</t>
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="F72" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G72" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G72" s="10" t="inlineStr">
+        <is>
+          <t>2018</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>Douglas Rauch</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr">
@@ -4118,14 +4118,14 @@
       </c>
       <c r="J72" s="10" t="inlineStr">
         <is>
-          <t>Consumer Defensi</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>UBSI</t>
+          <t>SFM</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
@@ -4135,43 +4135,43 @@
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>United Bankshares, Inc.</t>
+          <t>Sprouts Farmers Market, In</t>
         </is>
       </c>
       <c r="D73" s="11" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="E73" s="11" t="n">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G73" s="10" t="inlineStr">
-        <is>
-          <t>2003</t>
+        <v>1</v>
+      </c>
+      <c r="G73" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>J. Mcnamara,Michael Fitzgerald</t>
+          <t>Douglas Rauch</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr">
         <is>
-          <t>Sequoia Network</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J73" s="10" t="inlineStr">
         <is>
-          <t>Financial Servic</t>
+          <t>Consumer Defensi</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>UBSI</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
@@ -4181,43 +4181,43 @@
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group Ltd</t>
+          <t>United Bankshares, Inc.</t>
         </is>
       </c>
       <c r="D74" s="11" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="E74" s="11" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G74" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>J. Mcnamara,Michael Fitzgerald</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Sequoia Network</t>
         </is>
       </c>
       <c r="J74" s="10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financial Servic</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
@@ -4227,43 +4227,43 @@
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>Danaos Corporation</t>
+          <t>Woodside Energy Group Ltd</t>
         </is>
       </c>
       <c r="D75" s="11" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E75" s="11" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="F75" s="12" t="n">
         <v>1</v>
       </c>
       <c r="G75" s="10" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="H75" s="10" t="inlineStr">
         <is>
-          <t>Dimitris Vastarouchas</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="I75" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Office</t>
+          <t>Billionaire/Oligarch Veh</t>
         </is>
       </c>
       <c r="J75" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>RLXXF</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -4273,31 +4273,31 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>RELX PLC</t>
+          <t>Danaos Corporation</t>
         </is>
       </c>
       <c r="D76" s="11" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E76" s="11" t="n">
         <v>1</v>
-      </c>
-      <c r="E76" s="11" t="n">
-        <v>0.6</v>
       </c>
       <c r="F76" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G76" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>2005</t>
         </is>
       </c>
       <c r="H76" s="10" t="inlineStr">
         <is>
-          <t>Suzanne Wood</t>
+          <t>Dimitris Vastarouchas</t>
         </is>
       </c>
       <c r="I76" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Veh</t>
+          <t>Gulf/Royal Family Office</t>
         </is>
       </c>
       <c r="J76" s="10" t="inlineStr">
@@ -4461,10 +4461,10 @@
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>-5.5</v>
+        <v>-5.3</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F80" s="12" t="n">
         <v>1</v>
@@ -4606,10 +4606,10 @@
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>18.8</v>
+        <v>19.3</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>4.4</v>
+        <v>5.7</v>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F8" s="12" t="n">
         <v>0.9</v>
@@ -5695,7 +5695,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>25.1</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
@@ -5845,7 +5845,7 @@
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
@@ -5875,7 +5875,7 @@
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
@@ -5905,18 +5905,18 @@
         </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Gregory Landis</t>
+          <t>Andrew Crowley</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>H2O America</t>
+          <t>Markel Group</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -5931,22 +5931,22 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>MKL</t>
         </is>
       </c>
       <c r="F13" s="12" t="n">
-        <v>19.6</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>C. Wes Burton</t>
+          <t>Gregory Landis</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Vulcan Materials</t>
+          <t>H2O America</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -5961,17 +5961,17 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>VMC</t>
+          <t>HTO</t>
         </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>18.9</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Cynthia Hostetler</t>
+          <t>C. Wes Burton</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -5995,13 +5995,13 @@
         </is>
       </c>
       <c r="F15" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>David Clement</t>
+          <t>Cynthia Hostetler</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -6025,13 +6025,13 @@
         </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Denson Franklin</t>
+          <t>David Clement</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -6055,13 +6055,13 @@
         </is>
       </c>
       <c r="F17" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>George Willis</t>
+          <t>Denson Franklin</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -6085,13 +6085,13 @@
         </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>J. Hill</t>
+          <t>George Willis</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -6115,13 +6115,13 @@
         </is>
       </c>
       <c r="F19" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>J. Thomas Hill</t>
+          <t>J. Hill</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -6145,13 +6145,13 @@
         </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Jerry Perkins</t>
+          <t>J. Thomas Hill</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -6175,13 +6175,13 @@
         </is>
       </c>
       <c r="F21" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Mark Warren</t>
+          <t>Jerry Perkins</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -6205,13 +6205,13 @@
         </is>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Mary Carlisle</t>
+          <t>Mark Warren</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -6235,13 +6235,13 @@
         </is>
       </c>
       <c r="F23" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Thomas Fanning</t>
+          <t>Mary Carlisle</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -6265,18 +6265,18 @@
         </is>
       </c>
       <c r="F24" s="12" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Tatiana Mitrova</t>
+          <t>Thomas Fanning</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>SLB (Other Energy Services</t>
+          <t>Vulcan Materials</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -6291,22 +6291,22 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>VMC</t>
         </is>
       </c>
       <c r="F25" s="12" t="n">
-        <v>18.7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>John Baker</t>
+          <t>Tatiana Mitrova</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>FRP Holdings</t>
+          <t>SLB (Other Energy Services</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -6321,22 +6321,22 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>FRPH</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="F26" s="12" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Annalisa Jenkins</t>
+          <t>W. Conn</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>COMPASS Pathways</t>
+          <t>Charter Communications</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -6351,22 +6351,22 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="F27" s="12" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>W. Conn</t>
+          <t>John Baker</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Charter Communications</t>
+          <t>FRP Holdings</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -6381,22 +6381,22 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>FRPH</t>
         </is>
       </c>
       <c r="F28" s="12" t="n">
-        <v>18.3</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Andrew Crowley</t>
+          <t>Brandon Lewis</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Markel Group</t>
+          <t>Veon</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -6411,17 +6411,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>MKL</t>
+          <t>VEON</t>
         </is>
       </c>
       <c r="F29" s="12" t="n">
-        <v>18.1</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>Brandon Lewis</t>
+          <t>Duncan Perry</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Duncan Perry</t>
+          <t>Mary Kissel</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Veon</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -6471,22 +6471,22 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>VEON</t>
+          <t>QXO</t>
         </is>
       </c>
       <c r="F31" s="12" t="n">
-        <v>17.6</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Mary Kissel</t>
+          <t>Richard Mulligan</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>Sana Biotechnology</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -6501,22 +6501,22 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>QXO</t>
+          <t>SANA</t>
         </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Richard Mulligan</t>
+          <t>David Wright</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Sana Biotechnology</t>
+          <t>Rezolve Ai</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -6526,27 +6526,27 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>SANA</t>
+          <t>RZLVW</t>
         </is>
       </c>
       <c r="F33" s="12" t="n">
-        <v>16.6</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>David Wright</t>
+          <t>Danny Shepherd</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Rezolve Ai</t>
+          <t>Beazer Homes USA</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -6556,12 +6556,12 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>RZLVW</t>
+          <t>BZH</t>
         </is>
       </c>
       <c r="F34" s="12" t="n">
@@ -6571,12 +6571,12 @@
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Danny Shepherd</t>
+          <t>Michael Insulan</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Beazer Homes USA</t>
+          <t>Electra Battery Materials</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -6591,22 +6591,22 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>BZH</t>
+          <t>ELBM</t>
         </is>
       </c>
       <c r="F35" s="12" t="n">
-        <v>16.1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Michael Insulan</t>
+          <t>Derek Kan</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Electra Battery Materials</t>
+          <t>Toll Brothers</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -6621,11 +6621,11 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>ELBM</t>
+          <t>TOL</t>
         </is>
       </c>
       <c r="F36" s="12" t="n">
-        <v>16</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
@@ -6661,12 +6661,12 @@
     <row r="38" ht="14" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Derek Kan</t>
+          <t>James Nelson</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Toll Brothers</t>
+          <t>Global Net Lease</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -6681,22 +6681,22 @@
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>TOL</t>
+          <t>GNL</t>
         </is>
       </c>
       <c r="F38" s="12" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>James Nelson</t>
+          <t>Annalisa Jenkins</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Global Net Lease</t>
+          <t>COMPASS Pathways</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -6711,22 +6711,22 @@
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>GNL</t>
+          <t>CMPS</t>
         </is>
       </c>
       <c r="F39" s="12" t="n">
-        <v>14.2</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Christodoro</t>
+          <t>Joseph Flaim</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Iamgold</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -6736,27 +6736,27 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>XRXDW</t>
+          <t>IAG</t>
         </is>
       </c>
       <c r="F40" s="12" t="n">
-        <v>13.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Louis Pastor</t>
+          <t>Franz Humer</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Xerox</t>
+          <t>Allogene Therapeutics</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -6771,22 +6771,22 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>XRXDW</t>
+          <t>ALLO</t>
         </is>
       </c>
       <c r="F41" s="12" t="n">
-        <v>13.7</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Joseph Flaim</t>
+          <t>Meryl Hartzband</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Iamgold</t>
+          <t>Everest Group (Hamilton</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -6796,27 +6796,27 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>IAG</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="F42" s="12" t="n">
-        <v>13.3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Franz Humer</t>
+          <t>Wilbur Ross</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Allogene Therapeutics</t>
+          <t>Coya Therapeutics</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -6831,22 +6831,22 @@
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>ALLO</t>
+          <t>COYA</t>
         </is>
       </c>
       <c r="F43" s="12" t="n">
-        <v>13.2</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Meryl Hartzband</t>
+          <t>Jonathan Frates</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Everest Group (Hamilton</t>
+          <t>SandRidge Energy</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -6861,22 +6861,22 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F44" s="12" t="n">
-        <v>13</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Wilbur Ross</t>
+          <t>Nancy Dunlap</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Coya Therapeutics</t>
+          <t>SandRidge Energy</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -6891,22 +6891,22 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>Jonathan Frates</t>
+          <t>Bill Roeschlein</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>SandRidge Energy</t>
+          <t>Tigo Energy</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
@@ -6921,22 +6921,22 @@
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>TYGO</t>
         </is>
       </c>
       <c r="F46" s="12" t="n">
-        <v>12.1</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Nancy Dunlap</t>
+          <t>Kathleen Quirk</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>SandRidge Energy</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -6951,22 +6951,22 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="F47" s="12" t="n">
-        <v>12.1</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Bill Roeschlein</t>
+          <t>Wendy Teramoto</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Tigo Energy</t>
+          <t>The Greenbrier Companies</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -6981,22 +6981,22 @@
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>TYGO</t>
+          <t>GBX</t>
         </is>
       </c>
       <c r="F48" s="12" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Wendy Teramoto</t>
+          <t>Anthony Williams</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>The Greenbrier Companies</t>
+          <t>Akamai Technologies</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -7011,22 +7011,22 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>GBX</t>
+          <t>AKAM</t>
         </is>
       </c>
       <c r="F49" s="12" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Thierry Pilenko</t>
+          <t>Kelly Osborne</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>LanzaTech Global</t>
+          <t>Kinross Gold</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>LNZA</t>
+          <t>KGCRF</t>
         </is>
       </c>
       <c r="F50" s="12" t="n">
@@ -7051,12 +7051,12 @@
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>Kelly Osborne</t>
+          <t>Thierry Pilenko</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Kinross Gold</t>
+          <t>LanzaTech Global</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>KGCRF</t>
+          <t>LNZA</t>
         </is>
       </c>
       <c r="F51" s="12" t="n">
@@ -7081,12 +7081,12 @@
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Kathleen Quirk</t>
+          <t>Sandra Bell</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Dye &amp; Durham</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>DYNDF</t>
         </is>
       </c>
       <c r="F52" s="12" t="n">
@@ -7111,12 +7111,12 @@
     <row r="53" ht="14" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>Sandra Bell</t>
+          <t>Stephen Gunther</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Dye &amp; Durham</t>
+          <t>Shoulder Innovations</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -7131,22 +7131,22 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>DYNDF</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F53" s="12" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>Stephen Gunther</t>
+          <t>Kenneth Gunderman</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Shoulder Innovations</t>
+          <t>Uniti Group (Financial Servi</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -7156,12 +7156,12 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="F54" s="12" t="n">
@@ -7171,12 +7171,12 @@
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Kenneth Gunderman</t>
+          <t>Bryan Murphy</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Uniti Group (Financial Servi</t>
+          <t>Greenlight Capital Re</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -7191,22 +7191,22 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>GLRE</t>
         </is>
       </c>
       <c r="F55" s="12" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Bryan Murphy</t>
+          <t>Allan D. Schoening</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Greenlight Capital Re</t>
+          <t>Civeo</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -7221,22 +7221,22 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>GLRE</t>
+          <t>CVEO</t>
         </is>
       </c>
       <c r="F56" s="12" t="n">
-        <v>10.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Anthony Williams</t>
+          <t>Jeffrey Fox</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Akamai Technologies</t>
+          <t>Westrock Coffee</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -7251,52 +7251,52 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AKAM</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="F57" s="12" t="n">
-        <v>10.3</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Allan D. Schoening</t>
+          <t>Dominic Picone</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Civeo</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Public Company</t>
+          <t>PE/Buyout</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>CVEO</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="F58" s="12" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Jeffrey Fox</t>
+          <t>Brian Corvese</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Westrock Coffee</t>
+          <t>Agenus</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -7311,27 +7311,27 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>AGEN</t>
         </is>
       </c>
       <c r="F59" s="12" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Dominic Picone</t>
+          <t>Mohammad Abu-Ghazaleh</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>Fresh Del Monte Produce</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>PE/Buyout</t>
+          <t>Public Company</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
@@ -7341,22 +7341,22 @@
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="F60" s="12" t="n">
-        <v>9.6</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Brian Corvese</t>
+          <t>Jonathan Christodoro</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Agenus</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -7371,22 +7371,22 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AGEN</t>
+          <t>XRXDW</t>
         </is>
       </c>
       <c r="F61" s="12" t="n">
-        <v>9.4</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Mohammad Abu-Ghazaleh</t>
+          <t>Louis Pastor</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Fresh Del Monte Produce</t>
+          <t>Xerox</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -7396,16 +7396,16 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>XRXDW</t>
         </is>
       </c>
       <c r="F62" s="12" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
@@ -7501,12 +7501,12 @@
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Randle Reece</t>
+          <t>Sylvia Summers</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>AMN Healthcare Services</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -7521,22 +7521,22 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>AMN</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="F66" s="12" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Pam Kaufman</t>
+          <t>Randle Reece</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Paramount Skydance</t>
+          <t>AMN Healthcare Services</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -7551,22 +7551,22 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>PSKY</t>
+          <t>AMN</t>
         </is>
       </c>
       <c r="F67" s="12" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>Mark DiPaolo</t>
+          <t>Pam Kaufman</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Innoviva</t>
+          <t>Paramount Skydance</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -7581,22 +7581,22 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>PSKY</t>
         </is>
       </c>
       <c r="F68" s="12" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Sylvia Summers</t>
+          <t>David Allen</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -7611,22 +7611,22 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="F69" s="12" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>David Habachy</t>
+          <t>Mark DiPaolo</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Ring Energy</t>
+          <t>Innoviva</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -7641,22 +7641,22 @@
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>REI</t>
+          <t>INVA</t>
         </is>
       </c>
       <c r="F70" s="12" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>David Moradi</t>
+          <t>David Habachy</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>AudioEye</t>
+          <t>Ring Energy</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -7671,22 +7671,22 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>REI</t>
         </is>
       </c>
       <c r="F71" s="12" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>Tiago Miranda</t>
+          <t>David Moradi</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Atlas Lithium</t>
+          <t>AudioEye</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -7701,22 +7701,22 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>ATLX</t>
+          <t>AEYE</t>
         </is>
       </c>
       <c r="F72" s="12" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>David Allen</t>
+          <t>Randall Weisenburger</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -7731,11 +7731,11 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="F73" s="12" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
@@ -7765,18 +7765,18 @@
         </is>
       </c>
       <c r="F74" s="12" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>Charles Leykum</t>
+          <t>Tiago Miranda</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Talon Capital (SPAC</t>
+          <t>Atlas Lithium</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -7791,22 +7791,22 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>TLNC</t>
+          <t>ATLX</t>
         </is>
       </c>
       <c r="F75" s="12" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Tony Buffin</t>
+          <t>Charles Leykum</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>DFS Furniture</t>
+          <t>Talon Capital (SPAC</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -7821,22 +7821,22 @@
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>DFS.L</t>
+          <t>TLNC</t>
         </is>
       </c>
       <c r="F76" s="12" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>Randall Weisenburger</t>
+          <t>Tony Buffin</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>MP Materials</t>
+          <t>DFS Furniture</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>DFS.L</t>
         </is>
       </c>
       <c r="F77" s="12" t="n">
@@ -7921,12 +7921,12 @@
     <row r="80" ht="14" customHeight="1">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>Laura Duda</t>
+          <t>Oscar Iglesias</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>The Goodyear Tire &amp; Rubber</t>
+          <t>Codere Online Luxembourg</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>CDROW</t>
         </is>
       </c>
       <c r="F80" s="12" t="n">
@@ -7951,12 +7951,12 @@
     <row r="81" ht="14" customHeight="1">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Oscar Iglesias</t>
+          <t>Laura Duda</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Codere Online Luxembourg</t>
+          <t>The Goodyear Tire &amp; Rubber</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>CDROW</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="F81" s="12" t="n">
@@ -8065,18 +8065,18 @@
         </is>
       </c>
       <c r="F84" s="12" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>R. Cox</t>
+          <t>Rebecca Grossman-Cohen</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Terex</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -8091,22 +8091,22 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>NYT</t>
         </is>
       </c>
       <c r="F85" s="12" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>John Campbell</t>
+          <t>R. Cox</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Porch Group</t>
+          <t>Terex</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -8121,22 +8121,22 @@
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="F86" s="12" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Rebecca Grossman-Cohen</t>
+          <t>John Campbell</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Porch Group</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -8151,11 +8151,11 @@
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>NYT</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="F87" s="12" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="F89" s="12" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="90" ht="14" customHeight="1">
@@ -8281,12 +8281,12 @@
     <row r="92" ht="14" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>Michael Denham</t>
+          <t>Anelise Lara</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>National Bank of Canada (Mon</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -8301,22 +8301,22 @@
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="F92" s="12" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>Donald Dixon</t>
+          <t>Michael Denham</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Amprius Technologies</t>
+          <t>National Bank of Canada (Mon</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -8331,22 +8331,22 @@
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="F93" s="12" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>Anelise Lara</t>
+          <t>Donald Dixon</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>Amprius Technologies</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -8361,7 +8361,7 @@
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>AMPX</t>
         </is>
       </c>
       <c r="F94" s="12" t="n">
@@ -8401,12 +8401,12 @@
     <row r="96" ht="14" customHeight="1">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>Michael Dougherty</t>
+          <t>Chris Siu</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Polaris (Automotive</t>
+          <t>Aehr Test Systems</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -8421,22 +8421,22 @@
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>PII</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="F96" s="12" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Chris Siu</t>
+          <t>Michael Dougherty</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Aehr Test Systems</t>
+          <t>Polaris (Automotive</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -8451,22 +8451,22 @@
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>PII</t>
         </is>
       </c>
       <c r="F97" s="12" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>Alan Ferguson</t>
+          <t>Suzanne Wood</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Harbour Energy</t>
+          <t>RELX (Information Technology</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>HBR.L</t>
+          <t>RLXXF</t>
         </is>
       </c>
       <c r="F98" s="12" t="n">
@@ -8491,7 +8491,7 @@
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Alexander Krane</t>
+          <t>Alan Ferguson</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
@@ -8521,7 +8521,7 @@
     <row r="100" ht="14" customHeight="1">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Andrea Pinarel</t>
+          <t>Alexander Krane</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -8551,7 +8551,7 @@
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>David Kennedy</t>
+          <t>Andrea Pinarel</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
@@ -8581,7 +8581,7 @@
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>Feyyaz Etiz</t>
+          <t>David Kennedy</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
@@ -8611,7 +8611,7 @@
     <row r="103" ht="14" customHeight="1">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Gustavo Baquero</t>
+          <t>Feyyaz Etiz</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
@@ -8641,7 +8641,7 @@
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Linda Cook</t>
+          <t>Gustavo Baquero</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
@@ -8671,7 +8671,7 @@
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Michael Tuffin</t>
+          <t>Linda Cook</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
@@ -8701,7 +8701,7 @@
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Nathan Mauzy</t>
+          <t>Michael Tuffin</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
@@ -8731,12 +8731,12 @@
     <row r="107" ht="14" customHeight="1">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Raffaele Zagari</t>
+          <t>Nathan Mauzy</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Star Bulk Carriers</t>
+          <t>Harbour Energy</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -8751,22 +8751,22 @@
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>HBR.L</t>
         </is>
       </c>
       <c r="F107" s="12" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1">
       <c r="A108" s="10" t="inlineStr">
         <is>
-          <t>Douglas Rauch</t>
+          <t>Raffaele Zagari</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>Sprouts Farmers Market</t>
+          <t>Star Bulk Carriers</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>SFM</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="F108" s="12" t="n">
@@ -8791,12 +8791,12 @@
     <row r="109" ht="14" customHeight="1">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>Arnaud Breuillac</t>
+          <t>Douglas Rauch</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>Woodside Energy Group</t>
+          <t>Sprouts Farmers Market</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -8811,22 +8811,22 @@
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>WOPEF</t>
+          <t>SFM</t>
         </is>
       </c>
       <c r="F109" s="12" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="110" ht="14" customHeight="1">
       <c r="A110" s="10" t="inlineStr">
         <is>
-          <t>Dimitris Vastarouchas</t>
+          <t>Arnaud Breuillac</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Danaos</t>
+          <t>Woodside Energy Group</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -8836,27 +8836,27 @@
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>Gulf/Royal Family Offi</t>
+          <t>Billionaire/Oligarch V</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>WOPEF</t>
         </is>
       </c>
       <c r="F110" s="12" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>Peter Loscher</t>
+          <t>Dimitris Vastarouchas</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Telefónica</t>
+          <t>Danaos</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -8866,27 +8866,27 @@
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch V</t>
+          <t>Gulf/Royal Family Offi</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="F111" s="12" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="112" ht="14" customHeight="1">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>Jane O'Keeffe</t>
+          <t>Peter Loscher</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Bancroft Fund</t>
+          <t>Telefónica</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>BCV-PA</t>
+          <t>VIV</t>
         </is>
       </c>
       <c r="F112" s="12" t="n">
@@ -8911,12 +8911,12 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>Suzanne Wood</t>
+          <t>Jane O'Keeffe</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>RELX (Information Technology</t>
+          <t>Bancroft Fund</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
@@ -8931,11 +8931,11 @@
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>RLXXF</t>
+          <t>BCV-PA</t>
         </is>
       </c>
       <c r="F113" s="12" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="114" ht="14" customHeight="1">
@@ -9295,7 +9295,7 @@
         </is>
       </c>
       <c r="F125" s="12" t="n">
-        <v>-0.5</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="126" ht="14" customHeight="1">
@@ -9355,7 +9355,7 @@
         </is>
       </c>
       <c r="F127" s="12" t="n">
-        <v>-5.5</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="128" ht="14" customHeight="1">

</xml_diff>